<commit_message>
Replace all 3 toilets (supply & install) — updated scope per Justin
</commit_message>
<xml_diff>
--- a/docs/san-palo-circle-robert-bird/San-Palo-Circle-Budget.xlsx
+++ b/docs/san-palo-circle-robert-bird/San-Palo-Circle-Budget.xlsx
@@ -1133,11 +1133,11 @@
     <row r="24" ht="16" customHeight="1">
       <c r="A24" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Toilet set</t>
+          <t xml:space="preserve">  Toilet replacement (supply &amp; install)</t>
         </is>
       </c>
       <c r="B24" s="7" t="n">
-        <v>350</v>
+        <v>500</v>
       </c>
       <c r="C24" s="14" t="inlineStr">
         <is>
@@ -1145,7 +1145,7 @@
         </is>
       </c>
       <c r="D24" s="7" t="n">
-        <v>490</v>
+        <v>700</v>
       </c>
       <c r="E24" s="9" t="inlineStr"/>
     </row>
@@ -1175,11 +1175,11 @@
         </is>
       </c>
       <c r="B26" s="16" t="n">
-        <v>15700</v>
+        <v>15850</v>
       </c>
       <c r="C26" s="15" t="n"/>
       <c r="D26" s="16" t="n">
-        <v>21980</v>
+        <v>22190</v>
       </c>
       <c r="E26" s="15" t="n"/>
     </row>
@@ -1432,11 +1432,11 @@
     <row r="41" ht="16" customHeight="1">
       <c r="A41" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Toilet set</t>
+          <t xml:space="preserve">  Toilet replacement (supply &amp; install)</t>
         </is>
       </c>
       <c r="B41" s="11" t="n">
-        <v>300</v>
+        <v>500</v>
       </c>
       <c r="C41" s="12" t="inlineStr">
         <is>
@@ -1444,7 +1444,7 @@
         </is>
       </c>
       <c r="D41" s="11" t="n">
-        <v>420</v>
+        <v>700</v>
       </c>
       <c r="E41" s="13" t="inlineStr"/>
     </row>
@@ -1474,11 +1474,11 @@
         </is>
       </c>
       <c r="B43" s="16" t="n">
-        <v>11800</v>
+        <v>12000</v>
       </c>
       <c r="C43" s="15" t="n"/>
       <c r="D43" s="16" t="n">
-        <v>16520</v>
+        <v>16800</v>
       </c>
       <c r="E43" s="15" t="n"/>
     </row>
@@ -1731,11 +1731,11 @@
     <row r="58" ht="16" customHeight="1">
       <c r="A58" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Toilet set</t>
+          <t xml:space="preserve">  Toilet replacement (supply &amp; install)</t>
         </is>
       </c>
       <c r="B58" s="7" t="n">
-        <v>275</v>
+        <v>500</v>
       </c>
       <c r="C58" s="14" t="inlineStr">
         <is>
@@ -1743,7 +1743,7 @@
         </is>
       </c>
       <c r="D58" s="7" t="n">
-        <v>385</v>
+        <v>700</v>
       </c>
       <c r="E58" s="9" t="inlineStr"/>
     </row>
@@ -1773,11 +1773,11 @@
         </is>
       </c>
       <c r="B60" s="16" t="n">
-        <v>10000</v>
+        <v>10225</v>
       </c>
       <c r="C60" s="15" t="n"/>
       <c r="D60" s="16" t="n">
-        <v>14000</v>
+        <v>14315</v>
       </c>
       <c r="E60" s="15" t="n"/>
     </row>
@@ -3043,11 +3043,11 @@
         </is>
       </c>
       <c r="B138" s="23" t="n">
-        <v>140179</v>
+        <v>140754</v>
       </c>
       <c r="C138" s="22" t="n"/>
       <c r="D138" s="23" t="n">
-        <v>194350</v>
+        <v>195155</v>
       </c>
       <c r="E138" s="24" t="inlineStr">
         <is>
@@ -3065,7 +3065,7 @@
       <c r="B140" s="25" t="n"/>
       <c r="C140" s="25" t="n"/>
       <c r="D140" s="26" t="n">
-        <v>194350</v>
+        <v>195155</v>
       </c>
       <c r="E140" s="25" t="n"/>
     </row>
@@ -3078,7 +3078,7 @@
       <c r="B141" s="27" t="n"/>
       <c r="C141" s="27" t="n"/>
       <c r="D141" s="28" t="n">
-        <v>15950</v>
+        <v>16030</v>
       </c>
       <c r="E141" s="27" t="n"/>
     </row>
@@ -3091,7 +3091,7 @@
       <c r="B142" s="29" t="n"/>
       <c r="C142" s="29" t="n"/>
       <c r="D142" s="30" t="n">
-        <v>54171</v>
+        <v>54401</v>
       </c>
       <c r="E142" s="29" t="n"/>
     </row>
@@ -3104,7 +3104,7 @@
       <c r="B143" s="25" t="n"/>
       <c r="C143" s="25" t="n"/>
       <c r="D143" s="26" t="n">
-        <v>38221</v>
+        <v>38371</v>
       </c>
       <c r="E143" s="25" t="n"/>
     </row>
@@ -3318,11 +3318,11 @@
         </is>
       </c>
       <c r="B157" s="36" t="n">
-        <v>172879</v>
+        <v>173454</v>
       </c>
       <c r="C157" s="35" t="n"/>
       <c r="D157" s="36" t="n">
-        <v>240130</v>
+        <v>240935</v>
       </c>
       <c r="E157" s="35" t="n"/>
     </row>

</xml_diff>

<commit_message>
Add stair tread replacement 14x; drop fire/smoke/junk removal items per Justin
</commit_message>
<xml_diff>
--- a/docs/san-palo-circle-robert-bird/San-Palo-Circle-Budget.xlsx
+++ b/docs/san-palo-circle-robert-bird/San-Palo-Circle-Budget.xlsx
@@ -730,7 +730,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E170"/>
+  <dimension ref="A1:E171"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -866,1140 +866,1140 @@
       <c r="E8" s="9" t="inlineStr"/>
     </row>
     <row r="9" ht="18" customHeight="1">
-      <c r="A9" s="15" t="inlineStr">
+      <c r="A9" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Stair tread replacement — est. 14 treads @ $100/tread client price</t>
+        </is>
+      </c>
+      <c r="B9" s="7" t="n">
+        <v>1000</v>
+      </c>
+      <c r="C9" s="14" t="inlineStr">
+        <is>
+          <t>40%</t>
+        </is>
+      </c>
+      <c r="D9" s="7" t="n">
+        <v>1400</v>
+      </c>
+      <c r="E9" s="9" t="inlineStr">
+        <is>
+          <t>Verify stair count at site visit</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="6" customHeight="1">
+      <c r="A10" s="15" t="inlineStr">
         <is>
           <t xml:space="preserve">  ▶  FLOORING SUBTOTAL</t>
         </is>
       </c>
-      <c r="B9" s="16" t="n">
-        <v>10579</v>
-      </c>
-      <c r="C9" s="15" t="n"/>
-      <c r="D9" s="16" t="n">
-        <v>12910</v>
-      </c>
-      <c r="E9" s="15" t="n"/>
-    </row>
-    <row r="10" ht="6" customHeight="1">
-      <c r="A10" s="17" t="n"/>
-      <c r="B10" s="17" t="n"/>
-      <c r="C10" s="17" t="n"/>
-      <c r="D10" s="17" t="n"/>
-      <c r="E10" s="17" t="n"/>
+      <c r="B10" s="16" t="n">
+        <v>11579</v>
+      </c>
+      <c r="C10" s="15" t="n"/>
+      <c r="D10" s="16" t="n">
+        <v>14310</v>
+      </c>
+      <c r="E10" s="15" t="n"/>
     </row>
     <row r="11" ht="18" customHeight="1">
-      <c r="A11" s="4" t="inlineStr">
+      <c r="A11" s="17" t="n"/>
+      <c r="B11" s="17" t="n"/>
+      <c r="C11" s="17" t="n"/>
+      <c r="D11" s="17" t="n"/>
+      <c r="E11" s="17" t="n"/>
+    </row>
+    <row r="12" ht="16" customHeight="1">
+      <c r="A12" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve">  02 — BATHROOM 1 (MASTER) — Full Remodel</t>
         </is>
       </c>
-      <c r="B11" s="40" t="n"/>
-      <c r="C11" s="40" t="n"/>
-      <c r="D11" s="40" t="n"/>
-      <c r="E11" s="41" t="n"/>
-    </row>
-    <row r="12" ht="16" customHeight="1">
-      <c r="A12" s="6" t="inlineStr">
+      <c r="B12" s="40" t="n"/>
+      <c r="C12" s="40" t="n"/>
+      <c r="D12" s="40" t="n"/>
+      <c r="E12" s="41" t="n"/>
+    </row>
+    <row r="13" ht="16" customHeight="1">
+      <c r="A13" s="6" t="inlineStr">
         <is>
           <t xml:space="preserve">  Demo &amp; haul-off</t>
         </is>
       </c>
-      <c r="B12" s="7" t="n">
+      <c r="B13" s="7" t="n">
         <v>1200</v>
       </c>
-      <c r="C12" s="14" t="inlineStr">
-        <is>
-          <t>40%</t>
-        </is>
-      </c>
-      <c r="D12" s="7" t="n">
+      <c r="C13" s="14" t="inlineStr">
+        <is>
+          <t>40%</t>
+        </is>
+      </c>
+      <c r="D13" s="7" t="n">
         <v>1680</v>
       </c>
-      <c r="E12" s="9" t="inlineStr"/>
-    </row>
-    <row r="13" ht="16" customHeight="1">
-      <c r="A13" s="10" t="inlineStr">
+      <c r="E13" s="9" t="inlineStr"/>
+    </row>
+    <row r="14" ht="16" customHeight="1">
+      <c r="A14" s="10" t="inlineStr">
         <is>
           <t xml:space="preserve">  Cement board &amp; waterproofing (RedGuard)</t>
         </is>
       </c>
-      <c r="B13" s="11" t="n">
+      <c r="B14" s="11" t="n">
         <v>800</v>
       </c>
-      <c r="C13" s="12" t="inlineStr">
-        <is>
-          <t>40%</t>
-        </is>
-      </c>
-      <c r="D13" s="11" t="n">
+      <c r="C14" s="12" t="inlineStr">
+        <is>
+          <t>40%</t>
+        </is>
+      </c>
+      <c r="D14" s="11" t="n">
         <v>1120</v>
       </c>
-      <c r="E13" s="13" t="inlineStr"/>
-    </row>
-    <row r="14" ht="16" customHeight="1">
-      <c r="A14" s="6" t="inlineStr">
+      <c r="E14" s="13" t="inlineStr"/>
+    </row>
+    <row r="15" ht="16" customHeight="1">
+      <c r="A15" s="6" t="inlineStr">
         <is>
           <t xml:space="preserve">  Hot mop shower pan</t>
         </is>
       </c>
-      <c r="B14" s="7" t="n">
+      <c r="B15" s="7" t="n">
         <v>500</v>
       </c>
-      <c r="C14" s="14" t="inlineStr">
-        <is>
-          <t>40%</t>
-        </is>
-      </c>
-      <c r="D14" s="7" t="n">
+      <c r="C15" s="14" t="inlineStr">
+        <is>
+          <t>40%</t>
+        </is>
+      </c>
+      <c r="D15" s="7" t="n">
         <v>700</v>
       </c>
-      <c r="E14" s="9" t="inlineStr"/>
-    </row>
-    <row r="15" ht="16" customHeight="1">
-      <c r="A15" s="10" t="inlineStr">
+      <c r="E15" s="9" t="inlineStr"/>
+    </row>
+    <row r="16" ht="16" customHeight="1">
+      <c r="A16" s="10" t="inlineStr">
         <is>
           <t xml:space="preserve">  Tile labor (Jose)</t>
         </is>
       </c>
-      <c r="B15" s="11" t="n">
+      <c r="B16" s="11" t="n">
         <v>4000</v>
       </c>
-      <c r="C15" s="12" t="inlineStr">
-        <is>
-          <t>40%</t>
-        </is>
-      </c>
-      <c r="D15" s="11" t="n">
+      <c r="C16" s="12" t="inlineStr">
+        <is>
+          <t>40%</t>
+        </is>
+      </c>
+      <c r="D16" s="11" t="n">
         <v>5600</v>
       </c>
-      <c r="E15" s="13" t="inlineStr"/>
-    </row>
-    <row r="16" ht="16" customHeight="1">
-      <c r="A16" s="6" t="inlineStr">
+      <c r="E16" s="13" t="inlineStr"/>
+    </row>
+    <row r="17" ht="16" customHeight="1">
+      <c r="A17" s="6" t="inlineStr">
         <is>
           <t xml:space="preserve">  Tile material — allowance</t>
         </is>
       </c>
-      <c r="B16" s="7" t="n">
+      <c r="B17" s="7" t="n">
         <v>1500</v>
       </c>
-      <c r="C16" s="14" t="inlineStr">
-        <is>
-          <t>40%</t>
-        </is>
-      </c>
-      <c r="D16" s="7" t="n">
+      <c r="C17" s="14" t="inlineStr">
+        <is>
+          <t>40%</t>
+        </is>
+      </c>
+      <c r="D17" s="7" t="n">
         <v>2100</v>
       </c>
-      <c r="E16" s="9" t="inlineStr">
+      <c r="E17" s="9" t="inlineStr">
         <is>
           <t>Client-selected; allowance</t>
         </is>
       </c>
     </row>
-    <row r="17" ht="16" customHeight="1">
-      <c r="A17" s="10" t="inlineStr">
+    <row r="18" ht="16" customHeight="1">
+      <c r="A18" s="10" t="inlineStr">
         <is>
           <t xml:space="preserve">  Plumbing rough &amp; finish</t>
         </is>
       </c>
-      <c r="B17" s="11" t="n">
+      <c r="B18" s="11" t="n">
         <v>1200</v>
       </c>
-      <c r="C17" s="12" t="inlineStr">
-        <is>
-          <t>40%</t>
-        </is>
-      </c>
-      <c r="D17" s="11" t="n">
+      <c r="C18" s="12" t="inlineStr">
+        <is>
+          <t>40%</t>
+        </is>
+      </c>
+      <c r="D18" s="11" t="n">
         <v>1680</v>
       </c>
-      <c r="E17" s="13" t="inlineStr"/>
-    </row>
-    <row r="18" ht="16" customHeight="1">
-      <c r="A18" s="6" t="inlineStr">
+      <c r="E18" s="13" t="inlineStr"/>
+    </row>
+    <row r="19" ht="16" customHeight="1">
+      <c r="A19" s="6" t="inlineStr">
         <is>
           <t xml:space="preserve">  Vanity cabinet — allowance</t>
         </is>
       </c>
-      <c r="B18" s="7" t="n">
+      <c r="B19" s="7" t="n">
         <v>1200</v>
       </c>
-      <c r="C18" s="14" t="inlineStr">
-        <is>
-          <t>40%</t>
-        </is>
-      </c>
-      <c r="D18" s="7" t="n">
+      <c r="C19" s="14" t="inlineStr">
+        <is>
+          <t>40%</t>
+        </is>
+      </c>
+      <c r="D19" s="7" t="n">
         <v>1680</v>
       </c>
-      <c r="E18" s="9" t="inlineStr"/>
-    </row>
-    <row r="19" ht="16" customHeight="1">
-      <c r="A19" s="10" t="inlineStr">
+      <c r="E19" s="9" t="inlineStr"/>
+    </row>
+    <row r="20" ht="16" customHeight="1">
+      <c r="A20" s="10" t="inlineStr">
         <is>
           <t xml:space="preserve">  Countertop — allowance</t>
         </is>
       </c>
-      <c r="B19" s="11" t="n">
+      <c r="B20" s="11" t="n">
         <v>800</v>
       </c>
-      <c r="C19" s="12" t="inlineStr">
-        <is>
-          <t>40%</t>
-        </is>
-      </c>
-      <c r="D19" s="11" t="n">
+      <c r="C20" s="12" t="inlineStr">
+        <is>
+          <t>40%</t>
+        </is>
+      </c>
+      <c r="D20" s="11" t="n">
         <v>1120</v>
       </c>
-      <c r="E19" s="13" t="inlineStr"/>
-    </row>
-    <row r="20" ht="16" customHeight="1">
-      <c r="A20" s="6" t="inlineStr">
+      <c r="E20" s="13" t="inlineStr"/>
+    </row>
+    <row r="21" ht="16" customHeight="1">
+      <c r="A21" s="6" t="inlineStr">
         <is>
           <t xml:space="preserve">  Fixtures allowance (faucet, hardware)</t>
         </is>
       </c>
-      <c r="B20" s="7" t="n">
+      <c r="B21" s="7" t="n">
         <v>600</v>
       </c>
-      <c r="C20" s="14" t="inlineStr">
-        <is>
-          <t>40%</t>
-        </is>
-      </c>
-      <c r="D20" s="7" t="n">
+      <c r="C21" s="14" t="inlineStr">
+        <is>
+          <t>40%</t>
+        </is>
+      </c>
+      <c r="D21" s="7" t="n">
         <v>840</v>
       </c>
-      <c r="E20" s="9" t="inlineStr"/>
-    </row>
-    <row r="21" ht="16" customHeight="1">
-      <c r="A21" s="10" t="inlineStr">
+      <c r="E21" s="9" t="inlineStr"/>
+    </row>
+    <row r="22" ht="16" customHeight="1">
+      <c r="A22" s="10" t="inlineStr">
         <is>
           <t xml:space="preserve">  Frameless glass shower enclosure</t>
         </is>
       </c>
-      <c r="B21" s="11" t="n">
+      <c r="B22" s="11" t="n">
         <v>2500</v>
       </c>
-      <c r="C21" s="12" t="inlineStr">
-        <is>
-          <t>40%</t>
-        </is>
-      </c>
-      <c r="D21" s="11" t="n">
+      <c r="C22" s="12" t="inlineStr">
+        <is>
+          <t>40%</t>
+        </is>
+      </c>
+      <c r="D22" s="11" t="n">
         <v>3500</v>
       </c>
-      <c r="E21" s="13" t="inlineStr"/>
-    </row>
-    <row r="22" ht="16" customHeight="1">
-      <c r="A22" s="6" t="inlineStr">
+      <c r="E22" s="13" t="inlineStr"/>
+    </row>
+    <row r="23" ht="16" customHeight="1">
+      <c r="A23" s="6" t="inlineStr">
         <is>
           <t xml:space="preserve">  GFCI outlets (code required)</t>
         </is>
       </c>
-      <c r="B22" s="7" t="n">
+      <c r="B23" s="7" t="n">
         <v>300</v>
       </c>
-      <c r="C22" s="14" t="inlineStr">
-        <is>
-          <t>40%</t>
-        </is>
-      </c>
-      <c r="D22" s="7" t="n">
+      <c r="C23" s="14" t="inlineStr">
+        <is>
+          <t>40%</t>
+        </is>
+      </c>
+      <c r="D23" s="7" t="n">
         <v>420</v>
       </c>
-      <c r="E22" s="9" t="inlineStr"/>
-    </row>
-    <row r="23" ht="16" customHeight="1">
-      <c r="A23" s="10" t="inlineStr">
+      <c r="E23" s="9" t="inlineStr"/>
+    </row>
+    <row r="24" ht="16" customHeight="1">
+      <c r="A24" s="10" t="inlineStr">
         <is>
           <t xml:space="preserve">  Exhaust fan replacement</t>
         </is>
       </c>
-      <c r="B23" s="11" t="n">
+      <c r="B24" s="11" t="n">
         <v>350</v>
       </c>
-      <c r="C23" s="12" t="inlineStr">
-        <is>
-          <t>40%</t>
-        </is>
-      </c>
-      <c r="D23" s="11" t="n">
+      <c r="C24" s="12" t="inlineStr">
+        <is>
+          <t>40%</t>
+        </is>
+      </c>
+      <c r="D24" s="11" t="n">
         <v>490</v>
       </c>
-      <c r="E23" s="13" t="inlineStr"/>
-    </row>
-    <row r="24" ht="16" customHeight="1">
-      <c r="A24" s="6" t="inlineStr">
+      <c r="E24" s="13" t="inlineStr"/>
+    </row>
+    <row r="25" ht="16" customHeight="1">
+      <c r="A25" s="6" t="inlineStr">
         <is>
           <t xml:space="preserve">  Toilet replacement (supply &amp; install)</t>
         </is>
       </c>
-      <c r="B24" s="7" t="n">
+      <c r="B25" s="7" t="n">
         <v>500</v>
       </c>
-      <c r="C24" s="14" t="inlineStr">
-        <is>
-          <t>40%</t>
-        </is>
-      </c>
-      <c r="D24" s="7" t="n">
+      <c r="C25" s="14" t="inlineStr">
+        <is>
+          <t>40%</t>
+        </is>
+      </c>
+      <c r="D25" s="7" t="n">
         <v>700</v>
       </c>
-      <c r="E24" s="9" t="inlineStr"/>
-    </row>
-    <row r="25" ht="16" customHeight="1">
-      <c r="A25" s="10" t="inlineStr">
+      <c r="E25" s="9" t="inlineStr"/>
+    </row>
+    <row r="26" ht="18" customHeight="1">
+      <c r="A26" s="10" t="inlineStr">
         <is>
           <t xml:space="preserve">  Paint &amp; touch-up</t>
         </is>
       </c>
-      <c r="B25" s="11" t="n">
+      <c r="B26" s="11" t="n">
         <v>400</v>
       </c>
-      <c r="C25" s="12" t="inlineStr">
-        <is>
-          <t>40%</t>
-        </is>
-      </c>
-      <c r="D25" s="11" t="n">
+      <c r="C26" s="12" t="inlineStr">
+        <is>
+          <t>40%</t>
+        </is>
+      </c>
+      <c r="D26" s="11" t="n">
         <v>560</v>
       </c>
-      <c r="E25" s="13" t="inlineStr"/>
-    </row>
-    <row r="26" ht="18" customHeight="1">
-      <c r="A26" s="15" t="inlineStr">
+      <c r="E26" s="13" t="inlineStr"/>
+    </row>
+    <row r="27" ht="6" customHeight="1">
+      <c r="A27" s="15" t="inlineStr">
         <is>
           <t xml:space="preserve">  ▶  BATH 1 SUBTOTAL</t>
         </is>
       </c>
-      <c r="B26" s="16" t="n">
+      <c r="B27" s="16" t="n">
         <v>15850</v>
       </c>
-      <c r="C26" s="15" t="n"/>
-      <c r="D26" s="16" t="n">
+      <c r="C27" s="15" t="n"/>
+      <c r="D27" s="16" t="n">
         <v>22190</v>
       </c>
-      <c r="E26" s="15" t="n"/>
-    </row>
-    <row r="27" ht="6" customHeight="1">
-      <c r="A27" s="17" t="n"/>
-      <c r="B27" s="17" t="n"/>
-      <c r="C27" s="17" t="n"/>
-      <c r="D27" s="17" t="n"/>
-      <c r="E27" s="17" t="n"/>
+      <c r="E27" s="15" t="n"/>
     </row>
     <row r="28" ht="18" customHeight="1">
-      <c r="A28" s="4" t="inlineStr">
+      <c r="A28" s="17" t="n"/>
+      <c r="B28" s="17" t="n"/>
+      <c r="C28" s="17" t="n"/>
+      <c r="D28" s="17" t="n"/>
+      <c r="E28" s="17" t="n"/>
+    </row>
+    <row r="29" ht="16" customHeight="1">
+      <c r="A29" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve">  03 — BATHROOM 2 (SECONDARY) — Full Remodel</t>
         </is>
       </c>
-      <c r="B28" s="40" t="n"/>
-      <c r="C28" s="40" t="n"/>
-      <c r="D28" s="40" t="n"/>
-      <c r="E28" s="41" t="n"/>
-    </row>
-    <row r="29" ht="16" customHeight="1">
-      <c r="A29" s="10" t="inlineStr">
+      <c r="B29" s="40" t="n"/>
+      <c r="C29" s="40" t="n"/>
+      <c r="D29" s="40" t="n"/>
+      <c r="E29" s="41" t="n"/>
+    </row>
+    <row r="30" ht="16" customHeight="1">
+      <c r="A30" s="10" t="inlineStr">
         <is>
           <t xml:space="preserve">  Demo &amp; haul-off</t>
         </is>
       </c>
-      <c r="B29" s="11" t="n">
+      <c r="B30" s="11" t="n">
         <v>800</v>
       </c>
-      <c r="C29" s="12" t="inlineStr">
-        <is>
-          <t>40%</t>
-        </is>
-      </c>
-      <c r="D29" s="11" t="n">
+      <c r="C30" s="12" t="inlineStr">
+        <is>
+          <t>40%</t>
+        </is>
+      </c>
+      <c r="D30" s="11" t="n">
         <v>1120</v>
       </c>
-      <c r="E29" s="13" t="inlineStr"/>
-    </row>
-    <row r="30" ht="16" customHeight="1">
-      <c r="A30" s="6" t="inlineStr">
+      <c r="E30" s="13" t="inlineStr"/>
+    </row>
+    <row r="31" ht="16" customHeight="1">
+      <c r="A31" s="6" t="inlineStr">
         <is>
           <t xml:space="preserve">  Cement board &amp; waterproofing</t>
         </is>
       </c>
-      <c r="B30" s="7" t="n">
+      <c r="B31" s="7" t="n">
         <v>600</v>
       </c>
-      <c r="C30" s="14" t="inlineStr">
-        <is>
-          <t>40%</t>
-        </is>
-      </c>
-      <c r="D30" s="7" t="n">
+      <c r="C31" s="14" t="inlineStr">
+        <is>
+          <t>40%</t>
+        </is>
+      </c>
+      <c r="D31" s="7" t="n">
         <v>840</v>
       </c>
-      <c r="E30" s="9" t="inlineStr"/>
-    </row>
-    <row r="31" ht="16" customHeight="1">
-      <c r="A31" s="10" t="inlineStr">
+      <c r="E31" s="9" t="inlineStr"/>
+    </row>
+    <row r="32" ht="16" customHeight="1">
+      <c r="A32" s="10" t="inlineStr">
         <is>
           <t xml:space="preserve">  Hot mop shower pan</t>
         </is>
       </c>
-      <c r="B31" s="11" t="n">
+      <c r="B32" s="11" t="n">
         <v>450</v>
       </c>
-      <c r="C31" s="12" t="inlineStr">
-        <is>
-          <t>40%</t>
-        </is>
-      </c>
-      <c r="D31" s="11" t="n">
+      <c r="C32" s="12" t="inlineStr">
+        <is>
+          <t>40%</t>
+        </is>
+      </c>
+      <c r="D32" s="11" t="n">
         <v>630</v>
       </c>
-      <c r="E31" s="13" t="inlineStr"/>
-    </row>
-    <row r="32" ht="16" customHeight="1">
-      <c r="A32" s="6" t="inlineStr">
+      <c r="E32" s="13" t="inlineStr"/>
+    </row>
+    <row r="33" ht="16" customHeight="1">
+      <c r="A33" s="6" t="inlineStr">
         <is>
           <t xml:space="preserve">  Tile labor (Jose)</t>
         </is>
       </c>
-      <c r="B32" s="7" t="n">
+      <c r="B33" s="7" t="n">
         <v>3000</v>
       </c>
-      <c r="C32" s="14" t="inlineStr">
-        <is>
-          <t>40%</t>
-        </is>
-      </c>
-      <c r="D32" s="7" t="n">
+      <c r="C33" s="14" t="inlineStr">
+        <is>
+          <t>40%</t>
+        </is>
+      </c>
+      <c r="D33" s="7" t="n">
         <v>4200</v>
       </c>
-      <c r="E32" s="9" t="inlineStr"/>
-    </row>
-    <row r="33" ht="16" customHeight="1">
-      <c r="A33" s="10" t="inlineStr">
+      <c r="E33" s="9" t="inlineStr"/>
+    </row>
+    <row r="34" ht="16" customHeight="1">
+      <c r="A34" s="10" t="inlineStr">
         <is>
           <t xml:space="preserve">  Tile material — allowance</t>
         </is>
       </c>
-      <c r="B33" s="11" t="n">
+      <c r="B34" s="11" t="n">
         <v>1300</v>
       </c>
-      <c r="C33" s="12" t="inlineStr">
-        <is>
-          <t>40%</t>
-        </is>
-      </c>
-      <c r="D33" s="11" t="n">
+      <c r="C34" s="12" t="inlineStr">
+        <is>
+          <t>40%</t>
+        </is>
+      </c>
+      <c r="D34" s="11" t="n">
         <v>1820</v>
       </c>
-      <c r="E33" s="13" t="inlineStr"/>
-    </row>
-    <row r="34" ht="16" customHeight="1">
-      <c r="A34" s="6" t="inlineStr">
+      <c r="E34" s="13" t="inlineStr"/>
+    </row>
+    <row r="35" ht="16" customHeight="1">
+      <c r="A35" s="6" t="inlineStr">
         <is>
           <t xml:space="preserve">  Plumbing rough &amp; finish</t>
         </is>
       </c>
-      <c r="B34" s="7" t="n">
+      <c r="B35" s="7" t="n">
         <v>900</v>
       </c>
-      <c r="C34" s="14" t="inlineStr">
-        <is>
-          <t>40%</t>
-        </is>
-      </c>
-      <c r="D34" s="7" t="n">
+      <c r="C35" s="14" t="inlineStr">
+        <is>
+          <t>40%</t>
+        </is>
+      </c>
+      <c r="D35" s="7" t="n">
         <v>1260</v>
       </c>
-      <c r="E34" s="9" t="inlineStr"/>
-    </row>
-    <row r="35" ht="16" customHeight="1">
-      <c r="A35" s="10" t="inlineStr">
+      <c r="E35" s="9" t="inlineStr"/>
+    </row>
+    <row r="36" ht="16" customHeight="1">
+      <c r="A36" s="10" t="inlineStr">
         <is>
           <t xml:space="preserve">  Vanity cabinet — allowance</t>
         </is>
       </c>
-      <c r="B35" s="11" t="n">
+      <c r="B36" s="11" t="n">
         <v>800</v>
       </c>
-      <c r="C35" s="12" t="inlineStr">
-        <is>
-          <t>40%</t>
-        </is>
-      </c>
-      <c r="D35" s="11" t="n">
+      <c r="C36" s="12" t="inlineStr">
+        <is>
+          <t>40%</t>
+        </is>
+      </c>
+      <c r="D36" s="11" t="n">
         <v>1120</v>
       </c>
-      <c r="E35" s="13" t="inlineStr"/>
-    </row>
-    <row r="36" ht="16" customHeight="1">
-      <c r="A36" s="6" t="inlineStr">
+      <c r="E36" s="13" t="inlineStr"/>
+    </row>
+    <row r="37" ht="16" customHeight="1">
+      <c r="A37" s="6" t="inlineStr">
         <is>
           <t xml:space="preserve">  Countertop — allowance</t>
         </is>
       </c>
-      <c r="B36" s="7" t="n">
+      <c r="B37" s="7" t="n">
         <v>600</v>
       </c>
-      <c r="C36" s="14" t="inlineStr">
-        <is>
-          <t>40%</t>
-        </is>
-      </c>
-      <c r="D36" s="7" t="n">
+      <c r="C37" s="14" t="inlineStr">
+        <is>
+          <t>40%</t>
+        </is>
+      </c>
+      <c r="D37" s="7" t="n">
         <v>840</v>
       </c>
-      <c r="E36" s="9" t="inlineStr"/>
-    </row>
-    <row r="37" ht="16" customHeight="1">
-      <c r="A37" s="10" t="inlineStr">
+      <c r="E37" s="9" t="inlineStr"/>
+    </row>
+    <row r="38" ht="16" customHeight="1">
+      <c r="A38" s="10" t="inlineStr">
         <is>
           <t xml:space="preserve">  Fixtures allowance</t>
         </is>
       </c>
-      <c r="B37" s="11" t="n">
+      <c r="B38" s="11" t="n">
         <v>500</v>
       </c>
-      <c r="C37" s="12" t="inlineStr">
-        <is>
-          <t>40%</t>
-        </is>
-      </c>
-      <c r="D37" s="11" t="n">
+      <c r="C38" s="12" t="inlineStr">
+        <is>
+          <t>40%</t>
+        </is>
+      </c>
+      <c r="D38" s="11" t="n">
         <v>700</v>
       </c>
-      <c r="E37" s="13" t="inlineStr"/>
-    </row>
-    <row r="38" ht="16" customHeight="1">
-      <c r="A38" s="6" t="inlineStr">
+      <c r="E38" s="13" t="inlineStr"/>
+    </row>
+    <row r="39" ht="16" customHeight="1">
+      <c r="A39" s="6" t="inlineStr">
         <is>
           <t xml:space="preserve">  Frameless glass enclosure</t>
         </is>
       </c>
-      <c r="B38" s="7" t="n">
+      <c r="B39" s="7" t="n">
         <v>1800</v>
       </c>
-      <c r="C38" s="14" t="inlineStr">
-        <is>
-          <t>40%</t>
-        </is>
-      </c>
-      <c r="D38" s="7" t="n">
+      <c r="C39" s="14" t="inlineStr">
+        <is>
+          <t>40%</t>
+        </is>
+      </c>
+      <c r="D39" s="7" t="n">
         <v>2520</v>
       </c>
-      <c r="E38" s="9" t="inlineStr"/>
-    </row>
-    <row r="39" ht="16" customHeight="1">
-      <c r="A39" s="10" t="inlineStr">
+      <c r="E39" s="9" t="inlineStr"/>
+    </row>
+    <row r="40" ht="16" customHeight="1">
+      <c r="A40" s="10" t="inlineStr">
         <is>
           <t xml:space="preserve">  GFCI outlets</t>
         </is>
       </c>
-      <c r="B39" s="11" t="n">
+      <c r="B40" s="11" t="n">
         <v>200</v>
       </c>
-      <c r="C39" s="12" t="inlineStr">
-        <is>
-          <t>40%</t>
-        </is>
-      </c>
-      <c r="D39" s="11" t="n">
+      <c r="C40" s="12" t="inlineStr">
+        <is>
+          <t>40%</t>
+        </is>
+      </c>
+      <c r="D40" s="11" t="n">
         <v>280</v>
       </c>
-      <c r="E39" s="13" t="inlineStr"/>
-    </row>
-    <row r="40" ht="16" customHeight="1">
-      <c r="A40" s="6" t="inlineStr">
+      <c r="E40" s="13" t="inlineStr"/>
+    </row>
+    <row r="41" ht="16" customHeight="1">
+      <c r="A41" s="6" t="inlineStr">
         <is>
           <t xml:space="preserve">  Exhaust fan replacement</t>
         </is>
       </c>
-      <c r="B40" s="7" t="n">
+      <c r="B41" s="7" t="n">
         <v>250</v>
       </c>
-      <c r="C40" s="14" t="inlineStr">
-        <is>
-          <t>40%</t>
-        </is>
-      </c>
-      <c r="D40" s="7" t="n">
+      <c r="C41" s="14" t="inlineStr">
+        <is>
+          <t>40%</t>
+        </is>
+      </c>
+      <c r="D41" s="7" t="n">
         <v>350</v>
       </c>
-      <c r="E40" s="9" t="inlineStr"/>
-    </row>
-    <row r="41" ht="16" customHeight="1">
-      <c r="A41" s="10" t="inlineStr">
+      <c r="E41" s="9" t="inlineStr"/>
+    </row>
+    <row r="42" ht="16" customHeight="1">
+      <c r="A42" s="10" t="inlineStr">
         <is>
           <t xml:space="preserve">  Toilet replacement (supply &amp; install)</t>
         </is>
       </c>
-      <c r="B41" s="11" t="n">
+      <c r="B42" s="11" t="n">
         <v>500</v>
       </c>
-      <c r="C41" s="12" t="inlineStr">
-        <is>
-          <t>40%</t>
-        </is>
-      </c>
-      <c r="D41" s="11" t="n">
+      <c r="C42" s="12" t="inlineStr">
+        <is>
+          <t>40%</t>
+        </is>
+      </c>
+      <c r="D42" s="11" t="n">
         <v>700</v>
       </c>
-      <c r="E41" s="13" t="inlineStr"/>
-    </row>
-    <row r="42" ht="16" customHeight="1">
-      <c r="A42" s="6" t="inlineStr">
+      <c r="E42" s="13" t="inlineStr"/>
+    </row>
+    <row r="43" ht="18" customHeight="1">
+      <c r="A43" s="6" t="inlineStr">
         <is>
           <t xml:space="preserve">  Paint &amp; touch-up</t>
         </is>
       </c>
-      <c r="B42" s="7" t="n">
+      <c r="B43" s="7" t="n">
         <v>300</v>
       </c>
-      <c r="C42" s="14" t="inlineStr">
-        <is>
-          <t>40%</t>
-        </is>
-      </c>
-      <c r="D42" s="7" t="n">
+      <c r="C43" s="14" t="inlineStr">
+        <is>
+          <t>40%</t>
+        </is>
+      </c>
+      <c r="D43" s="7" t="n">
         <v>420</v>
       </c>
-      <c r="E42" s="9" t="inlineStr"/>
-    </row>
-    <row r="43" ht="18" customHeight="1">
-      <c r="A43" s="15" t="inlineStr">
+      <c r="E43" s="9" t="inlineStr"/>
+    </row>
+    <row r="44" ht="6" customHeight="1">
+      <c r="A44" s="15" t="inlineStr">
         <is>
           <t xml:space="preserve">  ▶  BATH 2 SUBTOTAL</t>
         </is>
       </c>
-      <c r="B43" s="16" t="n">
+      <c r="B44" s="16" t="n">
         <v>12000</v>
       </c>
-      <c r="C43" s="15" t="n"/>
-      <c r="D43" s="16" t="n">
+      <c r="C44" s="15" t="n"/>
+      <c r="D44" s="16" t="n">
         <v>16800</v>
       </c>
-      <c r="E43" s="15" t="n"/>
-    </row>
-    <row r="44" ht="6" customHeight="1">
-      <c r="A44" s="17" t="n"/>
-      <c r="B44" s="17" t="n"/>
-      <c r="C44" s="17" t="n"/>
-      <c r="D44" s="17" t="n"/>
-      <c r="E44" s="17" t="n"/>
+      <c r="E44" s="15" t="n"/>
     </row>
     <row r="45" ht="18" customHeight="1">
-      <c r="A45" s="4" t="inlineStr">
+      <c r="A45" s="17" t="n"/>
+      <c r="B45" s="17" t="n"/>
+      <c r="C45" s="17" t="n"/>
+      <c r="D45" s="17" t="n"/>
+      <c r="E45" s="17" t="n"/>
+    </row>
+    <row r="46" ht="16" customHeight="1">
+      <c r="A46" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve">  04 — BATHROOM 3 (HALL) — Full Remodel</t>
         </is>
       </c>
-      <c r="B45" s="40" t="n"/>
-      <c r="C45" s="40" t="n"/>
-      <c r="D45" s="40" t="n"/>
-      <c r="E45" s="41" t="n"/>
-    </row>
-    <row r="46" ht="16" customHeight="1">
-      <c r="A46" s="6" t="inlineStr">
+      <c r="B46" s="40" t="n"/>
+      <c r="C46" s="40" t="n"/>
+      <c r="D46" s="40" t="n"/>
+      <c r="E46" s="41" t="n"/>
+    </row>
+    <row r="47" ht="16" customHeight="1">
+      <c r="A47" s="6" t="inlineStr">
         <is>
           <t xml:space="preserve">  Demo &amp; haul-off</t>
         </is>
       </c>
-      <c r="B46" s="7" t="n">
+      <c r="B47" s="7" t="n">
         <v>600</v>
       </c>
-      <c r="C46" s="14" t="inlineStr">
-        <is>
-          <t>40%</t>
-        </is>
-      </c>
-      <c r="D46" s="7" t="n">
+      <c r="C47" s="14" t="inlineStr">
+        <is>
+          <t>40%</t>
+        </is>
+      </c>
+      <c r="D47" s="7" t="n">
         <v>840</v>
       </c>
-      <c r="E46" s="9" t="inlineStr"/>
-    </row>
-    <row r="47" ht="16" customHeight="1">
-      <c r="A47" s="10" t="inlineStr">
+      <c r="E47" s="9" t="inlineStr"/>
+    </row>
+    <row r="48" ht="16" customHeight="1">
+      <c r="A48" s="10" t="inlineStr">
         <is>
           <t xml:space="preserve">  Cement board &amp; waterproofing</t>
         </is>
       </c>
-      <c r="B47" s="11" t="n">
+      <c r="B48" s="11" t="n">
         <v>500</v>
       </c>
-      <c r="C47" s="12" t="inlineStr">
-        <is>
-          <t>40%</t>
-        </is>
-      </c>
-      <c r="D47" s="11" t="n">
+      <c r="C48" s="12" t="inlineStr">
+        <is>
+          <t>40%</t>
+        </is>
+      </c>
+      <c r="D48" s="11" t="n">
         <v>700</v>
       </c>
-      <c r="E47" s="13" t="inlineStr"/>
-    </row>
-    <row r="48" ht="16" customHeight="1">
-      <c r="A48" s="6" t="inlineStr">
+      <c r="E48" s="13" t="inlineStr"/>
+    </row>
+    <row r="49" ht="16" customHeight="1">
+      <c r="A49" s="6" t="inlineStr">
         <is>
           <t xml:space="preserve">  Hot mop shower pan</t>
         </is>
       </c>
-      <c r="B48" s="7" t="n">
+      <c r="B49" s="7" t="n">
         <v>400</v>
       </c>
-      <c r="C48" s="14" t="inlineStr">
-        <is>
-          <t>40%</t>
-        </is>
-      </c>
-      <c r="D48" s="7" t="n">
+      <c r="C49" s="14" t="inlineStr">
+        <is>
+          <t>40%</t>
+        </is>
+      </c>
+      <c r="D49" s="7" t="n">
         <v>560</v>
       </c>
-      <c r="E48" s="9" t="inlineStr"/>
-    </row>
-    <row r="49" ht="16" customHeight="1">
-      <c r="A49" s="10" t="inlineStr">
+      <c r="E49" s="9" t="inlineStr"/>
+    </row>
+    <row r="50" ht="16" customHeight="1">
+      <c r="A50" s="10" t="inlineStr">
         <is>
           <t xml:space="preserve">  Tile labor (Jose)</t>
         </is>
       </c>
-      <c r="B49" s="11" t="n">
+      <c r="B50" s="11" t="n">
         <v>2500</v>
       </c>
-      <c r="C49" s="12" t="inlineStr">
-        <is>
-          <t>40%</t>
-        </is>
-      </c>
-      <c r="D49" s="11" t="n">
+      <c r="C50" s="12" t="inlineStr">
+        <is>
+          <t>40%</t>
+        </is>
+      </c>
+      <c r="D50" s="11" t="n">
         <v>3500</v>
       </c>
-      <c r="E49" s="13" t="inlineStr"/>
-    </row>
-    <row r="50" ht="16" customHeight="1">
-      <c r="A50" s="6" t="inlineStr">
+      <c r="E50" s="13" t="inlineStr"/>
+    </row>
+    <row r="51" ht="16" customHeight="1">
+      <c r="A51" s="6" t="inlineStr">
         <is>
           <t xml:space="preserve">  Tile material — allowance</t>
         </is>
       </c>
-      <c r="B50" s="7" t="n">
+      <c r="B51" s="7" t="n">
         <v>1200</v>
       </c>
-      <c r="C50" s="14" t="inlineStr">
-        <is>
-          <t>40%</t>
-        </is>
-      </c>
-      <c r="D50" s="7" t="n">
+      <c r="C51" s="14" t="inlineStr">
+        <is>
+          <t>40%</t>
+        </is>
+      </c>
+      <c r="D51" s="7" t="n">
         <v>1680</v>
       </c>
-      <c r="E50" s="9" t="inlineStr"/>
-    </row>
-    <row r="51" ht="16" customHeight="1">
-      <c r="A51" s="10" t="inlineStr">
+      <c r="E51" s="9" t="inlineStr"/>
+    </row>
+    <row r="52" ht="16" customHeight="1">
+      <c r="A52" s="10" t="inlineStr">
         <is>
           <t xml:space="preserve">  Plumbing rough &amp; finish</t>
         </is>
       </c>
-      <c r="B51" s="11" t="n">
+      <c r="B52" s="11" t="n">
         <v>800</v>
       </c>
-      <c r="C51" s="12" t="inlineStr">
-        <is>
-          <t>40%</t>
-        </is>
-      </c>
-      <c r="D51" s="11" t="n">
+      <c r="C52" s="12" t="inlineStr">
+        <is>
+          <t>40%</t>
+        </is>
+      </c>
+      <c r="D52" s="11" t="n">
         <v>1120</v>
       </c>
-      <c r="E51" s="13" t="inlineStr"/>
-    </row>
-    <row r="52" ht="16" customHeight="1">
-      <c r="A52" s="6" t="inlineStr">
+      <c r="E52" s="13" t="inlineStr"/>
+    </row>
+    <row r="53" ht="16" customHeight="1">
+      <c r="A53" s="6" t="inlineStr">
         <is>
           <t xml:space="preserve">  Vanity cabinet — allowance</t>
         </is>
       </c>
-      <c r="B52" s="7" t="n">
+      <c r="B53" s="7" t="n">
         <v>700</v>
       </c>
-      <c r="C52" s="14" t="inlineStr">
-        <is>
-          <t>40%</t>
-        </is>
-      </c>
-      <c r="D52" s="7" t="n">
+      <c r="C53" s="14" t="inlineStr">
+        <is>
+          <t>40%</t>
+        </is>
+      </c>
+      <c r="D53" s="7" t="n">
         <v>980</v>
       </c>
-      <c r="E52" s="9" t="inlineStr"/>
-    </row>
-    <row r="53" ht="16" customHeight="1">
-      <c r="A53" s="10" t="inlineStr">
+      <c r="E53" s="9" t="inlineStr"/>
+    </row>
+    <row r="54" ht="16" customHeight="1">
+      <c r="A54" s="10" t="inlineStr">
         <is>
           <t xml:space="preserve">  Countertop — allowance</t>
         </is>
       </c>
-      <c r="B53" s="11" t="n">
+      <c r="B54" s="11" t="n">
         <v>500</v>
       </c>
-      <c r="C53" s="12" t="inlineStr">
-        <is>
-          <t>40%</t>
-        </is>
-      </c>
-      <c r="D53" s="11" t="n">
+      <c r="C54" s="12" t="inlineStr">
+        <is>
+          <t>40%</t>
+        </is>
+      </c>
+      <c r="D54" s="11" t="n">
         <v>700</v>
       </c>
-      <c r="E53" s="13" t="inlineStr"/>
-    </row>
-    <row r="54" ht="16" customHeight="1">
-      <c r="A54" s="6" t="inlineStr">
+      <c r="E54" s="13" t="inlineStr"/>
+    </row>
+    <row r="55" ht="16" customHeight="1">
+      <c r="A55" s="6" t="inlineStr">
         <is>
           <t xml:space="preserve">  Fixtures allowance</t>
         </is>
       </c>
-      <c r="B54" s="7" t="n">
+      <c r="B55" s="7" t="n">
         <v>400</v>
       </c>
-      <c r="C54" s="14" t="inlineStr">
-        <is>
-          <t>40%</t>
-        </is>
-      </c>
-      <c r="D54" s="7" t="n">
+      <c r="C55" s="14" t="inlineStr">
+        <is>
+          <t>40%</t>
+        </is>
+      </c>
+      <c r="D55" s="7" t="n">
         <v>560</v>
       </c>
-      <c r="E54" s="9" t="inlineStr"/>
-    </row>
-    <row r="55" ht="16" customHeight="1">
-      <c r="A55" s="10" t="inlineStr">
+      <c r="E55" s="9" t="inlineStr"/>
+    </row>
+    <row r="56" ht="16" customHeight="1">
+      <c r="A56" s="10" t="inlineStr">
         <is>
           <t xml:space="preserve">  Frameless glass door</t>
         </is>
       </c>
-      <c r="B55" s="11" t="n">
+      <c r="B56" s="11" t="n">
         <v>1500</v>
       </c>
-      <c r="C55" s="12" t="inlineStr">
-        <is>
-          <t>40%</t>
-        </is>
-      </c>
-      <c r="D55" s="11" t="n">
+      <c r="C56" s="12" t="inlineStr">
+        <is>
+          <t>40%</t>
+        </is>
+      </c>
+      <c r="D56" s="11" t="n">
         <v>2100</v>
       </c>
-      <c r="E55" s="13" t="inlineStr"/>
-    </row>
-    <row r="56" ht="16" customHeight="1">
-      <c r="A56" s="6" t="inlineStr">
+      <c r="E56" s="13" t="inlineStr"/>
+    </row>
+    <row r="57" ht="16" customHeight="1">
+      <c r="A57" s="6" t="inlineStr">
         <is>
           <t xml:space="preserve">  GFCI outlets</t>
         </is>
       </c>
-      <c r="B56" s="7" t="n">
+      <c r="B57" s="7" t="n">
         <v>150</v>
       </c>
-      <c r="C56" s="14" t="inlineStr">
-        <is>
-          <t>40%</t>
-        </is>
-      </c>
-      <c r="D56" s="7" t="n">
+      <c r="C57" s="14" t="inlineStr">
+        <is>
+          <t>40%</t>
+        </is>
+      </c>
+      <c r="D57" s="7" t="n">
         <v>210</v>
       </c>
-      <c r="E56" s="9" t="inlineStr"/>
-    </row>
-    <row r="57" ht="16" customHeight="1">
-      <c r="A57" s="10" t="inlineStr">
+      <c r="E57" s="9" t="inlineStr"/>
+    </row>
+    <row r="58" ht="16" customHeight="1">
+      <c r="A58" s="10" t="inlineStr">
         <is>
           <t xml:space="preserve">  Exhaust fan replacement</t>
         </is>
       </c>
-      <c r="B57" s="11" t="n">
+      <c r="B58" s="11" t="n">
         <v>200</v>
       </c>
-      <c r="C57" s="12" t="inlineStr">
-        <is>
-          <t>40%</t>
-        </is>
-      </c>
-      <c r="D57" s="11" t="n">
+      <c r="C58" s="12" t="inlineStr">
+        <is>
+          <t>40%</t>
+        </is>
+      </c>
+      <c r="D58" s="11" t="n">
         <v>280</v>
       </c>
-      <c r="E57" s="13" t="inlineStr"/>
-    </row>
-    <row r="58" ht="16" customHeight="1">
-      <c r="A58" s="6" t="inlineStr">
+      <c r="E58" s="13" t="inlineStr"/>
+    </row>
+    <row r="59" ht="16" customHeight="1">
+      <c r="A59" s="6" t="inlineStr">
         <is>
           <t xml:space="preserve">  Toilet replacement (supply &amp; install)</t>
         </is>
       </c>
-      <c r="B58" s="7" t="n">
+      <c r="B59" s="7" t="n">
         <v>500</v>
       </c>
-      <c r="C58" s="14" t="inlineStr">
-        <is>
-          <t>40%</t>
-        </is>
-      </c>
-      <c r="D58" s="7" t="n">
+      <c r="C59" s="14" t="inlineStr">
+        <is>
+          <t>40%</t>
+        </is>
+      </c>
+      <c r="D59" s="7" t="n">
         <v>700</v>
       </c>
-      <c r="E58" s="9" t="inlineStr"/>
-    </row>
-    <row r="59" ht="16" customHeight="1">
-      <c r="A59" s="10" t="inlineStr">
+      <c r="E59" s="9" t="inlineStr"/>
+    </row>
+    <row r="60" ht="18" customHeight="1">
+      <c r="A60" s="10" t="inlineStr">
         <is>
           <t xml:space="preserve">  Paint &amp; touch-up</t>
         </is>
       </c>
-      <c r="B59" s="11" t="n">
+      <c r="B60" s="11" t="n">
         <v>275</v>
       </c>
-      <c r="C59" s="12" t="inlineStr">
-        <is>
-          <t>40%</t>
-        </is>
-      </c>
-      <c r="D59" s="11" t="n">
+      <c r="C60" s="12" t="inlineStr">
+        <is>
+          <t>40%</t>
+        </is>
+      </c>
+      <c r="D60" s="11" t="n">
         <v>385</v>
       </c>
-      <c r="E59" s="13" t="inlineStr"/>
-    </row>
-    <row r="60" ht="18" customHeight="1">
-      <c r="A60" s="15" t="inlineStr">
+      <c r="E60" s="13" t="inlineStr"/>
+    </row>
+    <row r="61" ht="6" customHeight="1">
+      <c r="A61" s="15" t="inlineStr">
         <is>
           <t xml:space="preserve">  ▶  BATH 3 SUBTOTAL</t>
         </is>
       </c>
-      <c r="B60" s="16" t="n">
+      <c r="B61" s="16" t="n">
         <v>10225</v>
       </c>
-      <c r="C60" s="15" t="n"/>
-      <c r="D60" s="16" t="n">
+      <c r="C61" s="15" t="n"/>
+      <c r="D61" s="16" t="n">
         <v>14315</v>
       </c>
-      <c r="E60" s="15" t="n"/>
-    </row>
-    <row r="61" ht="6" customHeight="1">
-      <c r="A61" s="17" t="n"/>
-      <c r="B61" s="17" t="n"/>
-      <c r="C61" s="17" t="n"/>
-      <c r="D61" s="17" t="n"/>
-      <c r="E61" s="17" t="n"/>
+      <c r="E61" s="15" t="n"/>
     </row>
     <row r="62" ht="18" customHeight="1">
-      <c r="A62" s="4" t="inlineStr">
+      <c r="A62" s="17" t="n"/>
+      <c r="B62" s="17" t="n"/>
+      <c r="C62" s="17" t="n"/>
+      <c r="D62" s="17" t="n"/>
+      <c r="E62" s="17" t="n"/>
+    </row>
+    <row r="63" ht="16" customHeight="1">
+      <c r="A63" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve">  05 — DRYWALL &amp; PAINT (Whole House — Extensive Repairs + Full Paint)</t>
         </is>
       </c>
-      <c r="B62" s="40" t="n"/>
-      <c r="C62" s="40" t="n"/>
-      <c r="D62" s="40" t="n"/>
-      <c r="E62" s="41" t="n"/>
-    </row>
-    <row r="63" ht="16" customHeight="1">
-      <c r="A63" s="10" t="inlineStr">
+      <c r="B63" s="40" t="n"/>
+      <c r="C63" s="40" t="n"/>
+      <c r="D63" s="40" t="n"/>
+      <c r="E63" s="41" t="n"/>
+    </row>
+    <row r="64" ht="16" customHeight="1">
+      <c r="A64" s="10" t="inlineStr">
         <is>
           <t xml:space="preserve">  Demo — remove damaged/mold-compromised drywall sections</t>
         </is>
       </c>
-      <c r="B63" s="11" t="n">
+      <c r="B64" s="11" t="n">
         <v>1500</v>
       </c>
-      <c r="C63" s="12" t="inlineStr">
-        <is>
-          <t>40%</t>
-        </is>
-      </c>
-      <c r="D63" s="11" t="n">
+      <c r="C64" s="12" t="inlineStr">
+        <is>
+          <t>40%</t>
+        </is>
+      </c>
+      <c r="D64" s="11" t="n">
         <v>2100</v>
       </c>
-      <c r="E63" s="13" t="inlineStr">
+      <c r="E64" s="13" t="inlineStr">
         <is>
           <t>Incl. haul-off</t>
         </is>
       </c>
     </row>
-    <row r="64" ht="16" customHeight="1">
-      <c r="A64" s="6" t="inlineStr">
+    <row r="65" ht="16" customHeight="1">
+      <c r="A65" s="6" t="inlineStr">
         <is>
           <t xml:space="preserve">  Drywall materials (sheets, tape, mud, screws)</t>
         </is>
       </c>
-      <c r="B64" s="7" t="n">
+      <c r="B65" s="7" t="n">
         <v>3500</v>
       </c>
-      <c r="C64" s="14" t="inlineStr">
-        <is>
-          <t>40%</t>
-        </is>
-      </c>
-      <c r="D64" s="7" t="n">
+      <c r="C65" s="14" t="inlineStr">
+        <is>
+          <t>40%</t>
+        </is>
+      </c>
+      <c r="D65" s="7" t="n">
         <v>4900</v>
       </c>
-      <c r="E64" s="9" t="inlineStr"/>
-    </row>
-    <row r="65" ht="16" customHeight="1">
-      <c r="A65" s="10" t="inlineStr">
+      <c r="E65" s="9" t="inlineStr"/>
+    </row>
+    <row r="66" ht="16" customHeight="1">
+      <c r="A66" s="10" t="inlineStr">
         <is>
           <t xml:space="preserve">  Drywall hanging — full house patches + new sections</t>
         </is>
       </c>
-      <c r="B65" s="11" t="n">
+      <c r="B66" s="11" t="n">
         <v>3000</v>
       </c>
-      <c r="C65" s="12" t="inlineStr">
-        <is>
-          <t>40%</t>
-        </is>
-      </c>
-      <c r="D65" s="11" t="n">
+      <c r="C66" s="12" t="inlineStr">
+        <is>
+          <t>40%</t>
+        </is>
+      </c>
+      <c r="D66" s="11" t="n">
         <v>4200</v>
       </c>
-      <c r="E65" s="13" t="inlineStr"/>
-    </row>
-    <row r="66" ht="16" customHeight="1">
-      <c r="A66" s="6" t="inlineStr">
+      <c r="E66" s="13" t="inlineStr"/>
+    </row>
+    <row r="67" ht="16" customHeight="1">
+      <c r="A67" s="6" t="inlineStr">
         <is>
           <t xml:space="preserve">  Tape, mud &amp; finishing (3-coat)</t>
         </is>
       </c>
-      <c r="B66" s="7" t="n">
+      <c r="B67" s="7" t="n">
         <v>2500</v>
       </c>
-      <c r="C66" s="14" t="inlineStr">
-        <is>
-          <t>40%</t>
-        </is>
-      </c>
-      <c r="D66" s="7" t="n">
+      <c r="C67" s="14" t="inlineStr">
+        <is>
+          <t>40%</t>
+        </is>
+      </c>
+      <c r="D67" s="7" t="n">
         <v>3500</v>
       </c>
-      <c r="E66" s="9" t="inlineStr"/>
-    </row>
-    <row r="67" ht="16" customHeight="1">
-      <c r="A67" s="10" t="inlineStr">
+      <c r="E67" s="9" t="inlineStr"/>
+    </row>
+    <row r="68" ht="16" customHeight="1">
+      <c r="A68" s="10" t="inlineStr">
         <is>
           <t xml:space="preserve">  Texture match (skip trowel / smooth per room)</t>
         </is>
       </c>
-      <c r="B67" s="11" t="n">
+      <c r="B68" s="11" t="n">
         <v>1500</v>
       </c>
-      <c r="C67" s="12" t="inlineStr">
-        <is>
-          <t>40%</t>
-        </is>
-      </c>
-      <c r="D67" s="11" t="n">
+      <c r="C68" s="12" t="inlineStr">
+        <is>
+          <t>40%</t>
+        </is>
+      </c>
+      <c r="D68" s="11" t="n">
         <v>2100</v>
       </c>
-      <c r="E67" s="13" t="inlineStr"/>
-    </row>
-    <row r="68" ht="16" customHeight="1">
-      <c r="A68" s="6" t="inlineStr">
+      <c r="E68" s="13" t="inlineStr"/>
+    </row>
+    <row r="69" ht="16" customHeight="1">
+      <c r="A69" s="6" t="inlineStr">
         <is>
           <t xml:space="preserve">  Interior paint labor — full house + ceilings + closets</t>
         </is>
       </c>
-      <c r="B68" s="7" t="n">
+      <c r="B69" s="7" t="n">
         <v>5500</v>
       </c>
-      <c r="C68" s="14" t="inlineStr">
-        <is>
-          <t>40%</t>
-        </is>
-      </c>
-      <c r="D68" s="7" t="n">
+      <c r="C69" s="14" t="inlineStr">
+        <is>
+          <t>40%</t>
+        </is>
+      </c>
+      <c r="D69" s="7" t="n">
         <v>7700</v>
       </c>
-      <c r="E68" s="9" t="inlineStr"/>
-    </row>
-    <row r="69" ht="16" customHeight="1">
-      <c r="A69" s="10" t="inlineStr">
+      <c r="E69" s="9" t="inlineStr"/>
+    </row>
+    <row r="70" ht="18" customHeight="1">
+      <c r="A70" s="10" t="inlineStr">
         <is>
           <t xml:space="preserve">  Paint materials &amp; primer (Sherwin-Williams)</t>
         </is>
       </c>
-      <c r="B69" s="11" t="n">
+      <c r="B70" s="11" t="n">
         <v>1800</v>
       </c>
-      <c r="C69" s="12" t="inlineStr">
-        <is>
-          <t>40%</t>
-        </is>
-      </c>
-      <c r="D69" s="11" t="n">
+      <c r="C70" s="12" t="inlineStr">
+        <is>
+          <t>40%</t>
+        </is>
+      </c>
+      <c r="D70" s="11" t="n">
         <v>2520</v>
       </c>
-      <c r="E69" s="13" t="inlineStr"/>
-    </row>
-    <row r="70" ht="18" customHeight="1">
-      <c r="A70" s="15" t="inlineStr">
+      <c r="E70" s="13" t="inlineStr"/>
+    </row>
+    <row r="71" ht="6" customHeight="1">
+      <c r="A71" s="15" t="inlineStr">
         <is>
           <t xml:space="preserve">  ▶  DRYWALL &amp; PAINT SUBTOTAL</t>
         </is>
       </c>
-      <c r="B70" s="16" t="n">
+      <c r="B71" s="16" t="n">
         <v>19300</v>
       </c>
-      <c r="C70" s="15" t="n"/>
-      <c r="D70" s="16" t="n">
+      <c r="C71" s="15" t="n"/>
+      <c r="D71" s="16" t="n">
         <v>27020</v>
       </c>
-      <c r="E70" s="15" t="n"/>
-    </row>
-    <row r="71" ht="6" customHeight="1">
-      <c r="A71" s="17" t="n"/>
-      <c r="B71" s="17" t="n"/>
-      <c r="C71" s="17" t="n"/>
-      <c r="D71" s="17" t="n"/>
-      <c r="E71" s="17" t="n"/>
+      <c r="E71" s="15" t="n"/>
     </row>
     <row r="72" ht="18" customHeight="1">
-      <c r="A72" s="4" t="inlineStr">
+      <c r="A72" s="17" t="n"/>
+      <c r="B72" s="17" t="n"/>
+      <c r="C72" s="17" t="n"/>
+      <c r="D72" s="17" t="n"/>
+      <c r="E72" s="17" t="n"/>
+    </row>
+    <row r="73" ht="16" customHeight="1">
+      <c r="A73" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve">  06 — MOLD REMEDIATION ⚠️  (Active mold found in kitchen wall cavity — see photos)</t>
         </is>
       </c>
-      <c r="B72" s="40" t="n"/>
-      <c r="C72" s="40" t="n"/>
-      <c r="D72" s="40" t="n"/>
-      <c r="E72" s="41" t="n"/>
-    </row>
-    <row r="73" ht="16" customHeight="1">
-      <c r="A73" s="18" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Professional IEP testing &amp; assessment</t>
-        </is>
-      </c>
-      <c r="B73" s="19" t="n">
-        <v>500</v>
-      </c>
-      <c r="C73" s="20" t="inlineStr">
-        <is>
-          <t>40%</t>
-        </is>
-      </c>
-      <c r="D73" s="19" t="n">
-        <v>700</v>
-      </c>
-      <c r="E73" s="21" t="inlineStr">
-        <is>
-          <t>Required before work begins</t>
-        </is>
-      </c>
+      <c r="B73" s="40" t="n"/>
+      <c r="C73" s="40" t="n"/>
+      <c r="D73" s="40" t="n"/>
+      <c r="E73" s="41" t="n"/>
     </row>
     <row r="74" ht="16" customHeight="1">
       <c r="A74" s="18" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Containment, HEPA vacuum &amp; chemical remediation</t>
+          <t xml:space="preserve">  Professional IEP testing &amp; assessment</t>
         </is>
       </c>
       <c r="B74" s="19" t="n">
-        <v>3500</v>
+        <v>500</v>
       </c>
       <c r="C74" s="20" t="inlineStr">
         <is>
@@ -2007,22 +2007,22 @@
         </is>
       </c>
       <c r="D74" s="19" t="n">
-        <v>4900</v>
+        <v>700</v>
       </c>
       <c r="E74" s="21" t="inlineStr">
         <is>
-          <t>Licensed remediator</t>
+          <t>Required before work begins</t>
         </is>
       </c>
     </row>
     <row r="75" ht="16" customHeight="1">
       <c r="A75" s="18" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Anti-microbial treatment (Concrobium/BioBan)</t>
+          <t xml:space="preserve">  Containment, HEPA vacuum &amp; chemical remediation</t>
         </is>
       </c>
       <c r="B75" s="19" t="n">
-        <v>500</v>
+        <v>3500</v>
       </c>
       <c r="C75" s="20" t="inlineStr">
         <is>
@@ -2030,14 +2030,18 @@
         </is>
       </c>
       <c r="D75" s="19" t="n">
-        <v>700</v>
-      </c>
-      <c r="E75" s="21" t="inlineStr"/>
+        <v>4900</v>
+      </c>
+      <c r="E75" s="21" t="inlineStr">
+        <is>
+          <t>Licensed remediator</t>
+        </is>
+      </c>
     </row>
     <row r="76" ht="16" customHeight="1">
       <c r="A76" s="18" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Contaminated material certified disposal</t>
+          <t xml:space="preserve">  Anti-microbial treatment (Concrobium/BioBan)</t>
         </is>
       </c>
       <c r="B76" s="19" t="n">
@@ -2054,980 +2058,992 @@
       <c r="E76" s="21" t="inlineStr"/>
     </row>
     <row r="77" ht="18" customHeight="1">
-      <c r="A77" s="15" t="inlineStr">
+      <c r="A77" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Contaminated material certified disposal</t>
+        </is>
+      </c>
+      <c r="B77" s="19" t="n">
+        <v>500</v>
+      </c>
+      <c r="C77" s="20" t="inlineStr">
+        <is>
+          <t>40%</t>
+        </is>
+      </c>
+      <c r="D77" s="19" t="n">
+        <v>700</v>
+      </c>
+      <c r="E77" s="21" t="inlineStr"/>
+    </row>
+    <row r="78" ht="6" customHeight="1">
+      <c r="A78" s="15" t="inlineStr">
         <is>
           <t xml:space="preserve">  ▶  MOLD REMEDIATION SUBTOTAL</t>
         </is>
       </c>
-      <c r="B77" s="16" t="n">
+      <c r="B78" s="16" t="n">
         <v>5000</v>
       </c>
-      <c r="C77" s="15" t="n"/>
-      <c r="D77" s="16" t="n">
+      <c r="C78" s="15" t="n"/>
+      <c r="D78" s="16" t="n">
         <v>7000</v>
       </c>
-      <c r="E77" s="15" t="n"/>
-    </row>
-    <row r="78" ht="6" customHeight="1">
-      <c r="A78" s="17" t="n"/>
-      <c r="B78" s="17" t="n"/>
-      <c r="C78" s="17" t="n"/>
-      <c r="D78" s="17" t="n"/>
-      <c r="E78" s="17" t="n"/>
+      <c r="E78" s="15" t="n"/>
     </row>
     <row r="79" ht="18" customHeight="1">
-      <c r="A79" s="4" t="inlineStr">
+      <c r="A79" s="17" t="n"/>
+      <c r="B79" s="17" t="n"/>
+      <c r="C79" s="17" t="n"/>
+      <c r="D79" s="17" t="n"/>
+      <c r="E79" s="17" t="n"/>
+    </row>
+    <row r="80" ht="16" customHeight="1">
+      <c r="A80" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve">  07 — WINDOWS &amp; SLIDING DOORS (Milgard Dual-Pane Retrofit)</t>
         </is>
       </c>
-      <c r="B79" s="40" t="n"/>
-      <c r="C79" s="40" t="n"/>
-      <c r="D79" s="40" t="n"/>
-      <c r="E79" s="41" t="n"/>
-    </row>
-    <row r="80" ht="16" customHeight="1">
-      <c r="A80" s="6" t="inlineStr">
+      <c r="B80" s="40" t="n"/>
+      <c r="C80" s="40" t="n"/>
+      <c r="D80" s="40" t="n"/>
+      <c r="E80" s="41" t="n"/>
+    </row>
+    <row r="81" ht="16" customHeight="1">
+      <c r="A81" s="6" t="inlineStr">
         <is>
           <t xml:space="preserve">  Window material — est. 18 units × $500 (Milgard)</t>
         </is>
       </c>
-      <c r="B80" s="7" t="n">
+      <c r="B81" s="7" t="n">
         <v>9000</v>
       </c>
-      <c r="C80" s="14" t="inlineStr">
-        <is>
-          <t>40%</t>
-        </is>
-      </c>
-      <c r="D80" s="7" t="n">
+      <c r="C81" s="14" t="inlineStr">
+        <is>
+          <t>40%</t>
+        </is>
+      </c>
+      <c r="D81" s="7" t="n">
         <v>12600</v>
       </c>
-      <c r="E80" s="9" t="inlineStr">
+      <c r="E81" s="9" t="inlineStr">
         <is>
           <t>Verify count at site visit</t>
         </is>
       </c>
     </row>
-    <row r="81" ht="16" customHeight="1">
-      <c r="A81" s="10" t="inlineStr">
+    <row r="82" ht="16" customHeight="1">
+      <c r="A82" s="10" t="inlineStr">
         <is>
           <t xml:space="preserve">  Window retrofit installation — 18 units × $400</t>
         </is>
       </c>
-      <c r="B81" s="11" t="n">
+      <c r="B82" s="11" t="n">
         <v>7200</v>
       </c>
-      <c r="C81" s="12" t="inlineStr">
-        <is>
-          <t>40%</t>
-        </is>
-      </c>
-      <c r="D81" s="11" t="n">
+      <c r="C82" s="12" t="inlineStr">
+        <is>
+          <t>40%</t>
+        </is>
+      </c>
+      <c r="D82" s="11" t="n">
         <v>10080</v>
       </c>
-      <c r="E81" s="13" t="inlineStr">
+      <c r="E82" s="13" t="inlineStr">
         <is>
           <t>Incl. stucco patch per window</t>
         </is>
       </c>
     </row>
-    <row r="82" ht="16" customHeight="1">
-      <c r="A82" s="6" t="inlineStr">
+    <row r="83" ht="16" customHeight="1">
+      <c r="A83" s="6" t="inlineStr">
         <is>
           <t xml:space="preserve">  Sliding door material — 2 units × $1,200</t>
         </is>
       </c>
-      <c r="B82" s="7" t="n">
+      <c r="B83" s="7" t="n">
         <v>2400</v>
       </c>
-      <c r="C82" s="14" t="inlineStr">
-        <is>
-          <t>40%</t>
-        </is>
-      </c>
-      <c r="D82" s="7" t="n">
+      <c r="C83" s="14" t="inlineStr">
+        <is>
+          <t>40%</t>
+        </is>
+      </c>
+      <c r="D83" s="7" t="n">
         <v>3360</v>
       </c>
-      <c r="E82" s="9" t="inlineStr"/>
-    </row>
-    <row r="83" ht="16" customHeight="1">
-      <c r="A83" s="10" t="inlineStr">
+      <c r="E83" s="9" t="inlineStr"/>
+    </row>
+    <row r="84" ht="18" customHeight="1">
+      <c r="A84" s="10" t="inlineStr">
         <is>
           <t xml:space="preserve">  Sliding door installation — 2 units × $750</t>
         </is>
       </c>
-      <c r="B83" s="11" t="n">
+      <c r="B84" s="11" t="n">
         <v>1500</v>
       </c>
-      <c r="C83" s="12" t="inlineStr">
-        <is>
-          <t>40%</t>
-        </is>
-      </c>
-      <c r="D83" s="11" t="n">
+      <c r="C84" s="12" t="inlineStr">
+        <is>
+          <t>40%</t>
+        </is>
+      </c>
+      <c r="D84" s="11" t="n">
         <v>2100</v>
       </c>
-      <c r="E83" s="13" t="inlineStr"/>
-    </row>
-    <row r="84" ht="18" customHeight="1">
-      <c r="A84" s="15" t="inlineStr">
+      <c r="E84" s="13" t="inlineStr"/>
+    </row>
+    <row r="85" ht="6" customHeight="1">
+      <c r="A85" s="15" t="inlineStr">
         <is>
           <t xml:space="preserve">  ▶  WINDOWS &amp; DOORS SUBTOTAL</t>
         </is>
       </c>
-      <c r="B84" s="16" t="n">
+      <c r="B85" s="16" t="n">
         <v>20100</v>
       </c>
-      <c r="C84" s="15" t="n"/>
-      <c r="D84" s="16" t="n">
+      <c r="C85" s="15" t="n"/>
+      <c r="D85" s="16" t="n">
         <v>28140</v>
       </c>
-      <c r="E84" s="15" t="n"/>
-    </row>
-    <row r="85" ht="6" customHeight="1">
-      <c r="A85" s="17" t="n"/>
-      <c r="B85" s="17" t="n"/>
-      <c r="C85" s="17" t="n"/>
-      <c r="D85" s="17" t="n"/>
-      <c r="E85" s="17" t="n"/>
+      <c r="E85" s="15" t="n"/>
     </row>
     <row r="86" ht="18" customHeight="1">
-      <c r="A86" s="4" t="inlineStr">
+      <c r="A86" s="17" t="n"/>
+      <c r="B86" s="17" t="n"/>
+      <c r="C86" s="17" t="n"/>
+      <c r="D86" s="17" t="n"/>
+      <c r="E86" s="17" t="n"/>
+    </row>
+    <row r="87" ht="16" customHeight="1">
+      <c r="A87" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve">  08 — POPCORN CEILING SCRAPE + LIGHTING (Whole House)</t>
         </is>
       </c>
-      <c r="B86" s="40" t="n"/>
-      <c r="C86" s="40" t="n"/>
-      <c r="D86" s="40" t="n"/>
-      <c r="E86" s="41" t="n"/>
-    </row>
-    <row r="87" ht="16" customHeight="1">
-      <c r="A87" s="10" t="inlineStr">
+      <c r="B87" s="40" t="n"/>
+      <c r="C87" s="40" t="n"/>
+      <c r="D87" s="40" t="n"/>
+      <c r="E87" s="41" t="n"/>
+    </row>
+    <row r="88" ht="16" customHeight="1">
+      <c r="A88" s="10" t="inlineStr">
         <is>
           <t xml:space="preserve">  Asbestos pre-test — REQUIRED (pre-1980 home)</t>
         </is>
       </c>
-      <c r="B87" s="11" t="n">
+      <c r="B88" s="11" t="n">
         <v>500</v>
       </c>
-      <c r="C87" s="12" t="inlineStr">
-        <is>
-          <t>40%</t>
-        </is>
-      </c>
-      <c r="D87" s="11" t="n">
+      <c r="C88" s="12" t="inlineStr">
+        <is>
+          <t>40%</t>
+        </is>
+      </c>
+      <c r="D88" s="11" t="n">
         <v>700</v>
       </c>
-      <c r="E87" s="13" t="inlineStr">
+      <c r="E88" s="13" t="inlineStr">
         <is>
           <t>Must test before any scraping</t>
         </is>
       </c>
     </row>
-    <row r="88" ht="16" customHeight="1">
-      <c r="A88" s="6" t="inlineStr">
+    <row r="89" ht="16" customHeight="1">
+      <c r="A89" s="6" t="inlineStr">
         <is>
           <t xml:space="preserve">  Popcorn ceiling scrape — full house ~2,668 SF</t>
         </is>
       </c>
-      <c r="B88" s="7" t="n">
+      <c r="B89" s="7" t="n">
         <v>4000</v>
       </c>
-      <c r="C88" s="14" t="inlineStr">
-        <is>
-          <t>40%</t>
-        </is>
-      </c>
-      <c r="D88" s="7" t="n">
+      <c r="C89" s="14" t="inlineStr">
+        <is>
+          <t>40%</t>
+        </is>
+      </c>
+      <c r="D89" s="7" t="n">
         <v>5600</v>
       </c>
-      <c r="E88" s="9" t="inlineStr">
+      <c r="E89" s="9" t="inlineStr">
         <is>
           <t>Wet scrape method</t>
         </is>
       </c>
     </row>
-    <row r="89" ht="16" customHeight="1">
-      <c r="A89" s="10" t="inlineStr">
+    <row r="90" ht="16" customHeight="1">
+      <c r="A90" s="10" t="inlineStr">
         <is>
           <t xml:space="preserve">  Remove &amp; replace existing fixtures (~15 units)</t>
         </is>
       </c>
-      <c r="B89" s="11" t="n">
+      <c r="B90" s="11" t="n">
         <v>2000</v>
       </c>
-      <c r="C89" s="12" t="inlineStr">
-        <is>
-          <t>40%</t>
-        </is>
-      </c>
-      <c r="D89" s="11" t="n">
+      <c r="C90" s="12" t="inlineStr">
+        <is>
+          <t>40%</t>
+        </is>
+      </c>
+      <c r="D90" s="11" t="n">
         <v>2800</v>
       </c>
-      <c r="E89" s="13" t="inlineStr"/>
-    </row>
-    <row r="90" ht="16" customHeight="1">
-      <c r="A90" s="6" t="inlineStr">
+      <c r="E90" s="13" t="inlineStr"/>
+    </row>
+    <row r="91" ht="16" customHeight="1">
+      <c r="A91" s="6" t="inlineStr">
         <is>
           <t xml:space="preserve">  New recessed can lights — ~25 added throughout</t>
         </is>
       </c>
-      <c r="B90" s="7" t="n">
+      <c r="B91" s="7" t="n">
         <v>5000</v>
       </c>
-      <c r="C90" s="14" t="inlineStr">
-        <is>
-          <t>40%</t>
-        </is>
-      </c>
-      <c r="D90" s="7" t="n">
+      <c r="C91" s="14" t="inlineStr">
+        <is>
+          <t>40%</t>
+        </is>
+      </c>
+      <c r="D91" s="7" t="n">
         <v>7000</v>
       </c>
-      <c r="E90" s="9" t="inlineStr">
+      <c r="E91" s="9" t="inlineStr">
         <is>
           <t>Labor + fixtures incl.</t>
         </is>
       </c>
     </row>
-    <row r="91" ht="16" customHeight="1">
-      <c r="A91" s="10" t="inlineStr">
+    <row r="92" ht="16" customHeight="1">
+      <c r="A92" s="10" t="inlineStr">
         <is>
           <t xml:space="preserve">  Electrical — new circuits, switch boxes, dimmers</t>
         </is>
       </c>
-      <c r="B91" s="11" t="n">
+      <c r="B92" s="11" t="n">
         <v>2000</v>
       </c>
-      <c r="C91" s="12" t="inlineStr">
-        <is>
-          <t>40%</t>
-        </is>
-      </c>
-      <c r="D91" s="11" t="n">
+      <c r="C92" s="12" t="inlineStr">
+        <is>
+          <t>40%</t>
+        </is>
+      </c>
+      <c r="D92" s="11" t="n">
         <v>2800</v>
       </c>
-      <c r="E91" s="13" t="inlineStr"/>
-    </row>
-    <row r="92" ht="16" customHeight="1">
-      <c r="A92" s="6" t="inlineStr">
+      <c r="E92" s="13" t="inlineStr"/>
+    </row>
+    <row r="93" ht="18" customHeight="1">
+      <c r="A93" s="6" t="inlineStr">
         <is>
           <t xml:space="preserve">  Dimmer switches — select rooms</t>
         </is>
       </c>
-      <c r="B92" s="7" t="n">
+      <c r="B93" s="7" t="n">
         <v>600</v>
       </c>
-      <c r="C92" s="14" t="inlineStr">
-        <is>
-          <t>40%</t>
-        </is>
-      </c>
-      <c r="D92" s="7" t="n">
+      <c r="C93" s="14" t="inlineStr">
+        <is>
+          <t>40%</t>
+        </is>
+      </c>
+      <c r="D93" s="7" t="n">
         <v>840</v>
       </c>
-      <c r="E92" s="9" t="inlineStr"/>
-    </row>
-    <row r="93" ht="18" customHeight="1">
-      <c r="A93" s="15" t="inlineStr">
+      <c r="E93" s="9" t="inlineStr"/>
+    </row>
+    <row r="94" ht="6" customHeight="1">
+      <c r="A94" s="15" t="inlineStr">
         <is>
           <t xml:space="preserve">  ▶  CEILINGS &amp; LIGHTING SUBTOTAL</t>
         </is>
       </c>
-      <c r="B93" s="16" t="n">
+      <c r="B94" s="16" t="n">
         <v>14100</v>
       </c>
-      <c r="C93" s="15" t="n"/>
-      <c r="D93" s="16" t="n">
+      <c r="C94" s="15" t="n"/>
+      <c r="D94" s="16" t="n">
         <v>19740</v>
       </c>
-      <c r="E93" s="15" t="n"/>
-    </row>
-    <row r="94" ht="6" customHeight="1">
-      <c r="A94" s="17" t="n"/>
-      <c r="B94" s="17" t="n"/>
-      <c r="C94" s="17" t="n"/>
-      <c r="D94" s="17" t="n"/>
-      <c r="E94" s="17" t="n"/>
+      <c r="E94" s="15" t="n"/>
     </row>
     <row r="95" ht="18" customHeight="1">
-      <c r="A95" s="4" t="inlineStr">
+      <c r="A95" s="17" t="n"/>
+      <c r="B95" s="17" t="n"/>
+      <c r="C95" s="17" t="n"/>
+      <c r="D95" s="17" t="n"/>
+      <c r="E95" s="17" t="n"/>
+    </row>
+    <row r="96" ht="16" customHeight="1">
+      <c r="A96" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve">  09 — EXTERIOR — Upstairs Patio Iron Railing &amp; Deck Repair</t>
         </is>
       </c>
-      <c r="B95" s="40" t="n"/>
-      <c r="C95" s="40" t="n"/>
-      <c r="D95" s="40" t="n"/>
-      <c r="E95" s="41" t="n"/>
-    </row>
-    <row r="96" ht="16" customHeight="1">
-      <c r="A96" s="6" t="inlineStr">
+      <c r="B96" s="40" t="n"/>
+      <c r="C96" s="40" t="n"/>
+      <c r="D96" s="40" t="n"/>
+      <c r="E96" s="41" t="n"/>
+    </row>
+    <row r="97" ht="16" customHeight="1">
+      <c r="A97" s="6" t="inlineStr">
         <is>
           <t xml:space="preserve">  Custom iron railing — upstairs back patio</t>
         </is>
       </c>
-      <c r="B96" s="7" t="n">
+      <c r="B97" s="7" t="n">
         <v>2500</v>
       </c>
-      <c r="C96" s="14" t="inlineStr">
-        <is>
-          <t>40%</t>
-        </is>
-      </c>
-      <c r="D96" s="7" t="n">
+      <c r="C97" s="14" t="inlineStr">
+        <is>
+          <t>40%</t>
+        </is>
+      </c>
+      <c r="D97" s="7" t="n">
         <v>3500</v>
       </c>
-      <c r="E96" s="9" t="inlineStr">
+      <c r="E97" s="9" t="inlineStr">
         <is>
           <t>Per scope</t>
         </is>
       </c>
     </row>
-    <row r="97" ht="16" customHeight="1">
-      <c r="A97" s="10" t="inlineStr">
+    <row r="98" ht="16" customHeight="1">
+      <c r="A98" s="10" t="inlineStr">
         <is>
           <t xml:space="preserve">  Exterior deck board repair / replacement</t>
         </is>
       </c>
-      <c r="B97" s="11" t="n">
+      <c r="B98" s="11" t="n">
         <v>1800</v>
       </c>
-      <c r="C97" s="12" t="inlineStr">
-        <is>
-          <t>40%</t>
-        </is>
-      </c>
-      <c r="D97" s="11" t="n">
+      <c r="C98" s="12" t="inlineStr">
+        <is>
+          <t>40%</t>
+        </is>
+      </c>
+      <c r="D98" s="11" t="n">
         <v>2520</v>
       </c>
-      <c r="E97" s="13" t="inlineStr"/>
-    </row>
-    <row r="98" ht="16" customHeight="1">
-      <c r="A98" s="6" t="inlineStr">
+      <c r="E98" s="13" t="inlineStr"/>
+    </row>
+    <row r="99" ht="18" customHeight="1">
+      <c r="A99" s="6" t="inlineStr">
         <is>
           <t xml:space="preserve">  Deck stain &amp; weatherproofing</t>
         </is>
       </c>
-      <c r="B98" s="7" t="n">
+      <c r="B99" s="7" t="n">
         <v>600</v>
       </c>
-      <c r="C98" s="14" t="inlineStr">
-        <is>
-          <t>40%</t>
-        </is>
-      </c>
-      <c r="D98" s="7" t="n">
+      <c r="C99" s="14" t="inlineStr">
+        <is>
+          <t>40%</t>
+        </is>
+      </c>
+      <c r="D99" s="7" t="n">
         <v>840</v>
       </c>
-      <c r="E98" s="9" t="inlineStr"/>
-    </row>
-    <row r="99" ht="18" customHeight="1">
-      <c r="A99" s="15" t="inlineStr">
+      <c r="E99" s="9" t="inlineStr"/>
+    </row>
+    <row r="100" ht="6" customHeight="1">
+      <c r="A100" s="15" t="inlineStr">
         <is>
           <t xml:space="preserve">  ▶  EXTERIOR SUBTOTAL</t>
         </is>
       </c>
-      <c r="B99" s="16" t="n">
+      <c r="B100" s="16" t="n">
         <v>4900</v>
       </c>
-      <c r="C99" s="15" t="n"/>
-      <c r="D99" s="16" t="n">
+      <c r="C100" s="15" t="n"/>
+      <c r="D100" s="16" t="n">
         <v>6860</v>
       </c>
-      <c r="E99" s="15" t="n"/>
-    </row>
-    <row r="100" ht="6" customHeight="1">
-      <c r="A100" s="17" t="n"/>
-      <c r="B100" s="17" t="n"/>
-      <c r="C100" s="17" t="n"/>
-      <c r="D100" s="17" t="n"/>
-      <c r="E100" s="17" t="n"/>
+      <c r="E100" s="15" t="n"/>
     </row>
     <row r="101" ht="18" customHeight="1">
-      <c r="A101" s="4" t="inlineStr">
+      <c r="A101" s="17" t="n"/>
+      <c r="B101" s="17" t="n"/>
+      <c r="C101" s="17" t="n"/>
+      <c r="D101" s="17" t="n"/>
+      <c r="E101" s="17" t="n"/>
+    </row>
+    <row r="102" ht="16" customHeight="1">
+      <c r="A102" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve">  10 — ALL NEW TRIM (Baseboard, Door Casing, Window Casing — Full House)</t>
         </is>
       </c>
-      <c r="B101" s="40" t="n"/>
-      <c r="C101" s="40" t="n"/>
-      <c r="D101" s="40" t="n"/>
-      <c r="E101" s="41" t="n"/>
-    </row>
-    <row r="102" ht="16" customHeight="1">
-      <c r="A102" s="6" t="inlineStr">
+      <c r="B102" s="40" t="n"/>
+      <c r="C102" s="40" t="n"/>
+      <c r="D102" s="40" t="n"/>
+      <c r="E102" s="41" t="n"/>
+    </row>
+    <row r="103" ht="16" customHeight="1">
+      <c r="A103" s="6" t="inlineStr">
         <is>
           <t xml:space="preserve">  Baseboard material — est. 650 LF</t>
         </is>
       </c>
-      <c r="B102" s="7" t="n">
+      <c r="B103" s="7" t="n">
         <v>1500</v>
       </c>
-      <c r="C102" s="14" t="inlineStr">
-        <is>
-          <t>40%</t>
-        </is>
-      </c>
-      <c r="D102" s="7" t="n">
+      <c r="C103" s="14" t="inlineStr">
+        <is>
+          <t>40%</t>
+        </is>
+      </c>
+      <c r="D103" s="7" t="n">
         <v>2100</v>
       </c>
-      <c r="E102" s="9" t="inlineStr"/>
-    </row>
-    <row r="103" ht="16" customHeight="1">
-      <c r="A103" s="10" t="inlineStr">
+      <c r="E103" s="9" t="inlineStr"/>
+    </row>
+    <row r="104" ht="16" customHeight="1">
+      <c r="A104" s="10" t="inlineStr">
         <is>
           <t xml:space="preserve">  Door casing material — est. 30 doors × 2 sides</t>
         </is>
       </c>
-      <c r="B103" s="11" t="n">
+      <c r="B104" s="11" t="n">
         <v>1200</v>
       </c>
-      <c r="C103" s="12" t="inlineStr">
-        <is>
-          <t>40%</t>
-        </is>
-      </c>
-      <c r="D103" s="11" t="n">
+      <c r="C104" s="12" t="inlineStr">
+        <is>
+          <t>40%</t>
+        </is>
+      </c>
+      <c r="D104" s="11" t="n">
         <v>1680</v>
       </c>
-      <c r="E103" s="13" t="inlineStr"/>
-    </row>
-    <row r="104" ht="16" customHeight="1">
-      <c r="A104" s="6" t="inlineStr">
+      <c r="E104" s="13" t="inlineStr"/>
+    </row>
+    <row r="105" ht="16" customHeight="1">
+      <c r="A105" s="6" t="inlineStr">
         <is>
           <t xml:space="preserve">  Window casing material — 18 windows</t>
         </is>
       </c>
-      <c r="B104" s="7" t="n">
+      <c r="B105" s="7" t="n">
         <v>1000</v>
       </c>
-      <c r="C104" s="14" t="inlineStr">
-        <is>
-          <t>40%</t>
-        </is>
-      </c>
-      <c r="D104" s="7" t="n">
+      <c r="C105" s="14" t="inlineStr">
+        <is>
+          <t>40%</t>
+        </is>
+      </c>
+      <c r="D105" s="7" t="n">
         <v>1400</v>
       </c>
-      <c r="E104" s="9" t="inlineStr"/>
-    </row>
-    <row r="105" ht="16" customHeight="1">
-      <c r="A105" s="10" t="inlineStr">
+      <c r="E105" s="9" t="inlineStr"/>
+    </row>
+    <row r="106" ht="18" customHeight="1">
+      <c r="A106" s="10" t="inlineStr">
         <is>
           <t xml:space="preserve">  Trim installation labor (full house)</t>
         </is>
       </c>
-      <c r="B105" s="11" t="n">
+      <c r="B106" s="11" t="n">
         <v>4500</v>
       </c>
-      <c r="C105" s="12" t="inlineStr">
-        <is>
-          <t>40%</t>
-        </is>
-      </c>
-      <c r="D105" s="11" t="n">
+      <c r="C106" s="12" t="inlineStr">
+        <is>
+          <t>40%</t>
+        </is>
+      </c>
+      <c r="D106" s="11" t="n">
         <v>6300</v>
       </c>
-      <c r="E105" s="13" t="inlineStr"/>
-    </row>
-    <row r="106" ht="18" customHeight="1">
-      <c r="A106" s="15" t="inlineStr">
+      <c r="E106" s="13" t="inlineStr"/>
+    </row>
+    <row r="107" ht="6" customHeight="1">
+      <c r="A107" s="15" t="inlineStr">
         <is>
           <t xml:space="preserve">  ▶  TRIM SUBTOTAL</t>
         </is>
       </c>
-      <c r="B106" s="16" t="n">
+      <c r="B107" s="16" t="n">
         <v>8200</v>
       </c>
-      <c r="C106" s="15" t="n"/>
-      <c r="D106" s="16" t="n">
+      <c r="C107" s="15" t="n"/>
+      <c r="D107" s="16" t="n">
         <v>11480</v>
       </c>
-      <c r="E106" s="15" t="n"/>
-    </row>
-    <row r="107" ht="6" customHeight="1">
-      <c r="A107" s="17" t="n"/>
-      <c r="B107" s="17" t="n"/>
-      <c r="C107" s="17" t="n"/>
-      <c r="D107" s="17" t="n"/>
-      <c r="E107" s="17" t="n"/>
+      <c r="E107" s="15" t="n"/>
     </row>
     <row r="108" ht="18" customHeight="1">
-      <c r="A108" s="4" t="inlineStr">
+      <c r="A108" s="17" t="n"/>
+      <c r="B108" s="17" t="n"/>
+      <c r="C108" s="17" t="n"/>
+      <c r="D108" s="17" t="n"/>
+      <c r="E108" s="17" t="n"/>
+    </row>
+    <row r="109" ht="16" customHeight="1">
+      <c r="A109" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve">  11 — HVAC REGISTER &amp; RETURN COVERS (New Throughout)</t>
         </is>
       </c>
-      <c r="B108" s="40" t="n"/>
-      <c r="C108" s="40" t="n"/>
-      <c r="D108" s="40" t="n"/>
-      <c r="E108" s="41" t="n"/>
-    </row>
-    <row r="109" ht="16" customHeight="1">
-      <c r="A109" s="10" t="inlineStr">
+      <c r="B109" s="40" t="n"/>
+      <c r="C109" s="40" t="n"/>
+      <c r="D109" s="40" t="n"/>
+      <c r="E109" s="41" t="n"/>
+    </row>
+    <row r="110" ht="16" customHeight="1">
+      <c r="A110" s="10" t="inlineStr">
         <is>
           <t xml:space="preserve">  Supply register covers — est. 20 units</t>
         </is>
       </c>
-      <c r="B109" s="11" t="n">
+      <c r="B110" s="11" t="n">
         <v>500</v>
       </c>
-      <c r="C109" s="12" t="inlineStr">
-        <is>
-          <t>40%</t>
-        </is>
-      </c>
-      <c r="D109" s="11" t="n">
+      <c r="C110" s="12" t="inlineStr">
+        <is>
+          <t>40%</t>
+        </is>
+      </c>
+      <c r="D110" s="11" t="n">
         <v>700</v>
       </c>
-      <c r="E109" s="13" t="inlineStr"/>
-    </row>
-    <row r="110" ht="16" customHeight="1">
-      <c r="A110" s="6" t="inlineStr">
+      <c r="E110" s="13" t="inlineStr"/>
+    </row>
+    <row r="111" ht="16" customHeight="1">
+      <c r="A111" s="6" t="inlineStr">
         <is>
           <t xml:space="preserve">  Return air vent covers — est. 6 units</t>
         </is>
       </c>
-      <c r="B110" s="7" t="n">
+      <c r="B111" s="7" t="n">
         <v>300</v>
       </c>
-      <c r="C110" s="14" t="inlineStr">
-        <is>
-          <t>40%</t>
-        </is>
-      </c>
-      <c r="D110" s="7" t="n">
+      <c r="C111" s="14" t="inlineStr">
+        <is>
+          <t>40%</t>
+        </is>
+      </c>
+      <c r="D111" s="7" t="n">
         <v>420</v>
       </c>
-      <c r="E110" s="9" t="inlineStr"/>
-    </row>
-    <row r="111" ht="16" customHeight="1">
-      <c r="A111" s="10" t="inlineStr">
+      <c r="E111" s="9" t="inlineStr"/>
+    </row>
+    <row r="112" ht="18" customHeight="1">
+      <c r="A112" s="10" t="inlineStr">
         <is>
           <t xml:space="preserve">  Installation labor</t>
         </is>
       </c>
-      <c r="B111" s="11" t="n">
+      <c r="B112" s="11" t="n">
         <v>300</v>
       </c>
-      <c r="C111" s="12" t="inlineStr">
-        <is>
-          <t>40%</t>
-        </is>
-      </c>
-      <c r="D111" s="11" t="n">
+      <c r="C112" s="12" t="inlineStr">
+        <is>
+          <t>40%</t>
+        </is>
+      </c>
+      <c r="D112" s="11" t="n">
         <v>420</v>
       </c>
-      <c r="E111" s="13" t="inlineStr"/>
-    </row>
-    <row r="112" ht="18" customHeight="1">
-      <c r="A112" s="15" t="inlineStr">
+      <c r="E112" s="13" t="inlineStr"/>
+    </row>
+    <row r="113" ht="6" customHeight="1">
+      <c r="A113" s="15" t="inlineStr">
         <is>
           <t xml:space="preserve">  ▶  HVAC COVERS SUBTOTAL</t>
         </is>
       </c>
-      <c r="B112" s="16" t="n">
+      <c r="B113" s="16" t="n">
         <v>1100</v>
       </c>
-      <c r="C112" s="15" t="n"/>
-      <c r="D112" s="16" t="n">
+      <c r="C113" s="15" t="n"/>
+      <c r="D113" s="16" t="n">
         <v>1540</v>
       </c>
-      <c r="E112" s="15" t="n"/>
-    </row>
-    <row r="113" ht="6" customHeight="1">
-      <c r="A113" s="17" t="n"/>
-      <c r="B113" s="17" t="n"/>
-      <c r="C113" s="17" t="n"/>
-      <c r="D113" s="17" t="n"/>
-      <c r="E113" s="17" t="n"/>
+      <c r="E113" s="15" t="n"/>
     </row>
     <row r="114" ht="18" customHeight="1">
-      <c r="A114" s="4" t="inlineStr">
+      <c r="A114" s="17" t="n"/>
+      <c r="B114" s="17" t="n"/>
+      <c r="C114" s="17" t="n"/>
+      <c r="D114" s="17" t="n"/>
+      <c r="E114" s="17" t="n"/>
+    </row>
+    <row r="115" ht="16" customHeight="1">
+      <c r="A115" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve">  12 — ELECTRICAL PANEL &amp; SUBPANEL REBUILD</t>
         </is>
       </c>
-      <c r="B114" s="40" t="n"/>
-      <c r="C114" s="40" t="n"/>
-      <c r="D114" s="40" t="n"/>
-      <c r="E114" s="41" t="n"/>
-    </row>
-    <row r="115" ht="16" customHeight="1">
-      <c r="A115" s="10" t="inlineStr">
+      <c r="B115" s="40" t="n"/>
+      <c r="C115" s="40" t="n"/>
+      <c r="D115" s="40" t="n"/>
+      <c r="E115" s="41" t="n"/>
+    </row>
+    <row r="116" ht="16" customHeight="1">
+      <c r="A116" s="10" t="inlineStr">
         <is>
           <t xml:space="preserve">  Main panel replacement — 200A</t>
         </is>
       </c>
-      <c r="B115" s="11" t="n">
+      <c r="B116" s="11" t="n">
         <v>3500</v>
       </c>
-      <c r="C115" s="12" t="inlineStr">
-        <is>
-          <t>40%</t>
-        </is>
-      </c>
-      <c r="D115" s="11" t="n">
+      <c r="C116" s="12" t="inlineStr">
+        <is>
+          <t>40%</t>
+        </is>
+      </c>
+      <c r="D116" s="11" t="n">
         <v>4900</v>
       </c>
-      <c r="E115" s="13" t="inlineStr"/>
-    </row>
-    <row r="116" ht="16" customHeight="1">
-      <c r="A116" s="6" t="inlineStr">
+      <c r="E116" s="13" t="inlineStr"/>
+    </row>
+    <row r="117" ht="16" customHeight="1">
+      <c r="A117" s="6" t="inlineStr">
         <is>
           <t xml:space="preserve">  Subpanel replacement / rebuild</t>
         </is>
       </c>
-      <c r="B116" s="7" t="n">
+      <c r="B117" s="7" t="n">
         <v>1500</v>
       </c>
-      <c r="C116" s="14" t="inlineStr">
-        <is>
-          <t>40%</t>
-        </is>
-      </c>
-      <c r="D116" s="7" t="n">
+      <c r="C117" s="14" t="inlineStr">
+        <is>
+          <t>40%</t>
+        </is>
+      </c>
+      <c r="D117" s="7" t="n">
         <v>2100</v>
       </c>
-      <c r="E116" s="9" t="inlineStr"/>
-    </row>
-    <row r="117" ht="16" customHeight="1">
-      <c r="A117" s="10" t="inlineStr">
+      <c r="E117" s="9" t="inlineStr"/>
+    </row>
+    <row r="118" ht="16" customHeight="1">
+      <c r="A118" s="10" t="inlineStr">
         <is>
           <t xml:space="preserve">  Licensed electrician labor</t>
         </is>
       </c>
-      <c r="B117" s="11" t="n">
+      <c r="B118" s="11" t="n">
         <v>4500</v>
       </c>
-      <c r="C117" s="12" t="inlineStr">
-        <is>
-          <t>40%</t>
-        </is>
-      </c>
-      <c r="D117" s="11" t="n">
+      <c r="C118" s="12" t="inlineStr">
+        <is>
+          <t>40%</t>
+        </is>
+      </c>
+      <c r="D118" s="11" t="n">
         <v>6300</v>
       </c>
-      <c r="E117" s="13" t="inlineStr"/>
-    </row>
-    <row r="118" ht="16" customHeight="1">
-      <c r="A118" s="6" t="inlineStr">
+      <c r="E118" s="13" t="inlineStr"/>
+    </row>
+    <row r="119" ht="18" customHeight="1">
+      <c r="A119" s="6" t="inlineStr">
         <is>
           <t xml:space="preserve">  Permit &amp; inspection fee</t>
         </is>
       </c>
-      <c r="B118" s="7" t="n">
+      <c r="B119" s="7" t="n">
         <v>600</v>
       </c>
-      <c r="C118" s="14" t="inlineStr">
-        <is>
-          <t>40%</t>
-        </is>
-      </c>
-      <c r="D118" s="7" t="n">
+      <c r="C119" s="14" t="inlineStr">
+        <is>
+          <t>40%</t>
+        </is>
+      </c>
+      <c r="D119" s="7" t="n">
         <v>840</v>
       </c>
-      <c r="E118" s="9" t="inlineStr"/>
-    </row>
-    <row r="119" ht="18" customHeight="1">
-      <c r="A119" s="15" t="inlineStr">
+      <c r="E119" s="9" t="inlineStr"/>
+    </row>
+    <row r="120" ht="6" customHeight="1">
+      <c r="A120" s="15" t="inlineStr">
         <is>
           <t xml:space="preserve">  ▶  ELECTRICAL PANEL SUBTOTAL</t>
         </is>
       </c>
-      <c r="B119" s="16" t="n">
+      <c r="B120" s="16" t="n">
         <v>10100</v>
       </c>
-      <c r="C119" s="15" t="n"/>
-      <c r="D119" s="16" t="n">
+      <c r="C120" s="15" t="n"/>
+      <c r="D120" s="16" t="n">
         <v>14140</v>
       </c>
-      <c r="E119" s="15" t="n"/>
-    </row>
-    <row r="120" ht="6" customHeight="1">
-      <c r="A120" s="17" t="n"/>
-      <c r="B120" s="17" t="n"/>
-      <c r="C120" s="17" t="n"/>
-      <c r="D120" s="17" t="n"/>
-      <c r="E120" s="17" t="n"/>
+      <c r="E120" s="15" t="n"/>
     </row>
     <row r="121" ht="18" customHeight="1">
-      <c r="A121" s="4" t="inlineStr">
+      <c r="A121" s="17" t="n"/>
+      <c r="B121" s="17" t="n"/>
+      <c r="C121" s="17" t="n"/>
+      <c r="D121" s="17" t="n"/>
+      <c r="E121" s="17" t="n"/>
+    </row>
+    <row r="122" ht="16" customHeight="1">
+      <c r="A122" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve">  13 — PLUMBING — External Drain Relocation</t>
         </is>
       </c>
-      <c r="B121" s="40" t="n"/>
-      <c r="C121" s="40" t="n"/>
-      <c r="D121" s="40" t="n"/>
-      <c r="E121" s="41" t="n"/>
-    </row>
-    <row r="122" ht="16" customHeight="1">
-      <c r="A122" s="6" t="inlineStr">
+      <c r="B122" s="40" t="n"/>
+      <c r="C122" s="40" t="n"/>
+      <c r="D122" s="40" t="n"/>
+      <c r="E122" s="41" t="n"/>
+    </row>
+    <row r="123" ht="16" customHeight="1">
+      <c r="A123" s="6" t="inlineStr">
         <is>
           <t xml:space="preserve">  Drain video camera inspection</t>
         </is>
       </c>
-      <c r="B122" s="7" t="n">
+      <c r="B123" s="7" t="n">
         <v>500</v>
       </c>
-      <c r="C122" s="14" t="inlineStr">
-        <is>
-          <t>40%</t>
-        </is>
-      </c>
-      <c r="D122" s="7" t="n">
+      <c r="C123" s="14" t="inlineStr">
+        <is>
+          <t>40%</t>
+        </is>
+      </c>
+      <c r="D123" s="7" t="n">
         <v>700</v>
       </c>
-      <c r="E122" s="9" t="inlineStr">
+      <c r="E123" s="9" t="inlineStr">
         <is>
           <t>Required before underground work</t>
         </is>
       </c>
     </row>
-    <row r="123" ht="16" customHeight="1">
-      <c r="A123" s="10" t="inlineStr">
+    <row r="124" ht="16" customHeight="1">
+      <c r="A124" s="10" t="inlineStr">
         <is>
           <t xml:space="preserve">  Excavation — external drain area</t>
         </is>
       </c>
-      <c r="B123" s="11" t="n">
+      <c r="B124" s="11" t="n">
         <v>2000</v>
       </c>
-      <c r="C123" s="12" t="inlineStr">
-        <is>
-          <t>40%</t>
-        </is>
-      </c>
-      <c r="D123" s="11" t="n">
+      <c r="C124" s="12" t="inlineStr">
+        <is>
+          <t>40%</t>
+        </is>
+      </c>
+      <c r="D124" s="11" t="n">
         <v>2800</v>
       </c>
-      <c r="E123" s="13" t="inlineStr"/>
-    </row>
-    <row r="124" ht="16" customHeight="1">
-      <c r="A124" s="6" t="inlineStr">
+      <c r="E124" s="13" t="inlineStr"/>
+    </row>
+    <row r="125" ht="16" customHeight="1">
+      <c r="A125" s="6" t="inlineStr">
         <is>
           <t xml:space="preserve">  Relocate drain pipe underground</t>
         </is>
       </c>
-      <c r="B124" s="7" t="n">
+      <c r="B125" s="7" t="n">
         <v>2500</v>
       </c>
-      <c r="C124" s="14" t="inlineStr">
-        <is>
-          <t>40%</t>
-        </is>
-      </c>
-      <c r="D124" s="7" t="n">
+      <c r="C125" s="14" t="inlineStr">
+        <is>
+          <t>40%</t>
+        </is>
+      </c>
+      <c r="D125" s="7" t="n">
         <v>3500</v>
       </c>
-      <c r="E124" s="9" t="inlineStr"/>
-    </row>
-    <row r="125" ht="16" customHeight="1">
-      <c r="A125" s="10" t="inlineStr">
+      <c r="E125" s="9" t="inlineStr"/>
+    </row>
+    <row r="126" ht="16" customHeight="1">
+      <c r="A126" s="10" t="inlineStr">
         <is>
           <t xml:space="preserve">  Tap into main drain line</t>
         </is>
       </c>
-      <c r="B125" s="11" t="n">
+      <c r="B126" s="11" t="n">
         <v>1500</v>
       </c>
-      <c r="C125" s="12" t="inlineStr">
-        <is>
-          <t>40%</t>
-        </is>
-      </c>
-      <c r="D125" s="11" t="n">
+      <c r="C126" s="12" t="inlineStr">
+        <is>
+          <t>40%</t>
+        </is>
+      </c>
+      <c r="D126" s="11" t="n">
         <v>2100</v>
       </c>
-      <c r="E125" s="13" t="inlineStr"/>
-    </row>
-    <row r="126" ht="16" customHeight="1">
-      <c r="A126" s="6" t="inlineStr">
+      <c r="E126" s="13" t="inlineStr"/>
+    </row>
+    <row r="127" ht="16" customHeight="1">
+      <c r="A127" s="6" t="inlineStr">
         <is>
           <t xml:space="preserve">  Backfill, compact &amp; surface restore</t>
         </is>
       </c>
-      <c r="B126" s="7" t="n">
+      <c r="B127" s="7" t="n">
         <v>600</v>
       </c>
-      <c r="C126" s="14" t="inlineStr">
-        <is>
-          <t>40%</t>
-        </is>
-      </c>
-      <c r="D126" s="7" t="n">
+      <c r="C127" s="14" t="inlineStr">
+        <is>
+          <t>40%</t>
+        </is>
+      </c>
+      <c r="D127" s="7" t="n">
         <v>840</v>
       </c>
-      <c r="E126" s="9" t="inlineStr"/>
-    </row>
-    <row r="127" ht="16" customHeight="1">
-      <c r="A127" s="10" t="inlineStr">
+      <c r="E127" s="9" t="inlineStr"/>
+    </row>
+    <row r="128" ht="16" customHeight="1">
+      <c r="A128" s="10" t="inlineStr">
         <is>
           <t xml:space="preserve">  Permit</t>
         </is>
       </c>
-      <c r="B127" s="11" t="n">
+      <c r="B128" s="11" t="n">
         <v>400</v>
       </c>
-      <c r="C127" s="12" t="inlineStr">
-        <is>
-          <t>40%</t>
-        </is>
-      </c>
-      <c r="D127" s="11" t="n">
+      <c r="C128" s="12" t="inlineStr">
+        <is>
+          <t>40%</t>
+        </is>
+      </c>
+      <c r="D128" s="11" t="n">
         <v>560</v>
       </c>
-      <c r="E127" s="13" t="inlineStr"/>
-    </row>
-    <row r="128" ht="16" customHeight="1">
-      <c r="A128" s="18" t="inlineStr">
+      <c r="E128" s="13" t="inlineStr"/>
+    </row>
+    <row r="129" ht="18" customHeight="1">
+      <c r="A129" s="18" t="inlineStr">
         <is>
           <t xml:space="preserve">  ⚠️  Main drain line repair — TBD post-camera</t>
         </is>
       </c>
-      <c r="B128" s="19" t="n">
+      <c r="B129" s="19" t="n">
         <v>0</v>
       </c>
-      <c r="C128" s="20" t="inlineStr">
+      <c r="C129" s="20" t="inlineStr">
         <is>
           <t>TBD</t>
         </is>
       </c>
-      <c r="D128" s="19" t="n">
+      <c r="D129" s="19" t="n">
         <v>0</v>
       </c>
-      <c r="E128" s="21" t="inlineStr">
+      <c r="E129" s="21" t="inlineStr">
         <is>
           <t>Homeowner flagged issues — CO on discovery</t>
         </is>
       </c>
     </row>
-    <row r="129" ht="18" customHeight="1">
-      <c r="A129" s="15" t="inlineStr">
+    <row r="130" ht="6" customHeight="1">
+      <c r="A130" s="15" t="inlineStr">
         <is>
           <t xml:space="preserve">  ▶  PLUMBING SUBTOTAL (excl. TBD drain)</t>
         </is>
       </c>
-      <c r="B129" s="16" t="n">
+      <c r="B130" s="16" t="n">
         <v>7500</v>
       </c>
-      <c r="C129" s="15" t="n"/>
-      <c r="D129" s="16" t="n">
+      <c r="C130" s="15" t="n"/>
+      <c r="D130" s="16" t="n">
         <v>10500</v>
       </c>
-      <c r="E129" s="15" t="n"/>
-    </row>
-    <row r="130" ht="6" customHeight="1">
-      <c r="A130" s="17" t="n"/>
-      <c r="B130" s="17" t="n"/>
-      <c r="C130" s="17" t="n"/>
-      <c r="D130" s="17" t="n"/>
-      <c r="E130" s="17" t="n"/>
+      <c r="E130" s="15" t="n"/>
     </row>
     <row r="131" ht="18" customHeight="1">
-      <c r="A131" s="4" t="inlineStr">
+      <c r="A131" s="17" t="n"/>
+      <c r="B131" s="17" t="n"/>
+      <c r="C131" s="17" t="n"/>
+      <c r="D131" s="17" t="n"/>
+      <c r="E131" s="17" t="n"/>
+    </row>
+    <row r="132" ht="16" customHeight="1">
+      <c r="A132" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve">  14 — ADDITIONAL ITEMS (Photo Findings + CA Rental Compliance)</t>
         </is>
       </c>
-      <c r="B131" s="40" t="n"/>
-      <c r="C131" s="40" t="n"/>
-      <c r="D131" s="40" t="n"/>
-      <c r="E131" s="41" t="n"/>
-    </row>
-    <row r="132" ht="16" customHeight="1">
-      <c r="A132" s="6" t="inlineStr">
+      <c r="B132" s="40" t="n"/>
+      <c r="C132" s="40" t="n"/>
+      <c r="D132" s="40" t="n"/>
+      <c r="E132" s="41" t="n"/>
+    </row>
+    <row r="133" ht="16" customHeight="1">
+      <c r="A133" s="6" t="inlineStr">
         <is>
           <t xml:space="preserve">  Smoke / CO detectors — full house (CA law)</t>
         </is>
       </c>
-      <c r="B132" s="7" t="n">
+      <c r="B133" s="7" t="n">
         <v>600</v>
       </c>
-      <c r="C132" s="14" t="inlineStr">
-        <is>
-          <t>40%</t>
-        </is>
-      </c>
-      <c r="D132" s="7" t="n">
+      <c r="C133" s="14" t="inlineStr">
+        <is>
+          <t>40%</t>
+        </is>
+      </c>
+      <c r="D133" s="7" t="n">
         <v>840</v>
       </c>
-      <c r="E132" s="9" t="inlineStr">
+      <c r="E133" s="9" t="inlineStr">
         <is>
           <t>Required for rental</t>
         </is>
       </c>
     </row>
-    <row r="133" ht="16" customHeight="1">
-      <c r="A133" s="10" t="inlineStr">
+    <row r="134" ht="16" customHeight="1">
+      <c r="A134" s="10" t="inlineStr">
         <is>
           <t xml:space="preserve">  Fireplace surround tile — complete unfinished work</t>
         </is>
       </c>
-      <c r="B133" s="11" t="n">
+      <c r="B134" s="11" t="n">
         <v>800</v>
       </c>
-      <c r="C133" s="12" t="inlineStr">
-        <is>
-          <t>40%</t>
-        </is>
-      </c>
-      <c r="D133" s="11" t="n">
+      <c r="C134" s="12" t="inlineStr">
+        <is>
+          <t>40%</t>
+        </is>
+      </c>
+      <c r="D134" s="11" t="n">
         <v>1120</v>
       </c>
-      <c r="E133" s="13" t="inlineStr">
+      <c r="E134" s="13" t="inlineStr">
         <is>
           <t>Incomplete per photos</t>
         </is>
       </c>
     </row>
-    <row r="134" ht="16" customHeight="1">
-      <c r="A134" s="6" t="inlineStr">
+    <row r="135" ht="16" customHeight="1">
+      <c r="A135" s="6" t="inlineStr">
         <is>
           <t xml:space="preserve">  Garage — close open electrical boxes + cover plates</t>
         </is>
       </c>
-      <c r="B134" s="7" t="n">
+      <c r="B135" s="7" t="n">
         <v>400</v>
       </c>
-      <c r="C134" s="14" t="inlineStr">
-        <is>
-          <t>40%</t>
-        </is>
-      </c>
-      <c r="D134" s="7" t="n">
+      <c r="C135" s="14" t="inlineStr">
+        <is>
+          <t>40%</t>
+        </is>
+      </c>
+      <c r="D135" s="7" t="n">
         <v>560</v>
       </c>
-      <c r="E134" s="9" t="inlineStr">
+      <c r="E135" s="9" t="inlineStr">
         <is>
           <t>Safety item per photos</t>
         </is>
       </c>
     </row>
-    <row r="135" ht="16" customHeight="1">
-      <c r="A135" s="15" t="inlineStr">
+    <row r="136" ht="18" customHeight="1">
+      <c r="A136" s="15" t="inlineStr">
         <is>
           <t xml:space="preserve">  ▶  ADDITIONAL ITEMS SUBTOTAL</t>
         </is>
       </c>
-      <c r="B135" s="16" t="n">
+      <c r="B136" s="16" t="n">
         <v>1800</v>
       </c>
-      <c r="C135" s="15" t="n"/>
-      <c r="D135" s="16" t="n">
+      <c r="C136" s="15" t="n"/>
+      <c r="D136" s="16" t="n">
         <v>2520</v>
       </c>
-      <c r="E135" s="15" t="n"/>
-    </row>
-    <row r="136" ht="18" customHeight="1">
-      <c r="A136" s="17" t="n"/>
-      <c r="B136" s="17" t="n"/>
-      <c r="C136" s="17" t="n"/>
-      <c r="D136" s="17" t="n"/>
-      <c r="E136" s="17" t="n"/>
+      <c r="E136" s="15" t="n"/>
     </row>
     <row r="137" ht="6" customHeight="1">
       <c r="A137" s="17" t="n"/>
@@ -3037,322 +3053,318 @@
       <c r="E137" s="17" t="n"/>
     </row>
     <row r="138" ht="6" customHeight="1">
-      <c r="A138" s="22" t="inlineStr">
+      <c r="A138" s="17" t="n"/>
+      <c r="B138" s="17" t="n"/>
+      <c r="C138" s="17" t="n"/>
+      <c r="D138" s="17" t="n"/>
+      <c r="E138" s="17" t="n"/>
+    </row>
+    <row r="139" ht="28" customHeight="1">
+      <c r="A139" s="22" t="inlineStr">
         <is>
           <t xml:space="preserve">  ★  PROJECT TOTAL (excluding optional kitchen)</t>
         </is>
       </c>
-      <c r="B138" s="23" t="n">
-        <v>140754</v>
-      </c>
-      <c r="C138" s="22" t="n"/>
-      <c r="D138" s="23" t="n">
-        <v>195155</v>
-      </c>
-      <c r="E138" s="24" t="inlineStr">
+      <c r="B139" s="23" t="n">
+        <v>141754</v>
+      </c>
+      <c r="C139" s="22" t="n"/>
+      <c r="D139" s="23" t="n">
+        <v>196555</v>
+      </c>
+      <c r="E139" s="24" t="inlineStr">
         <is>
           <t>+ TBD: Main drain line repair</t>
         </is>
       </c>
     </row>
-    <row r="139" ht="28" customHeight="1"/>
-    <row r="140">
-      <c r="A140" s="25" t="inlineStr">
+    <row r="140"/>
+    <row r="141" ht="18" customHeight="1">
+      <c r="A141" s="25" t="inlineStr">
         <is>
           <t xml:space="preserve">  Total Client Charge</t>
         </is>
       </c>
-      <c r="B140" s="25" t="n"/>
-      <c r="C140" s="25" t="n"/>
-      <c r="D140" s="26" t="n">
-        <v>195155</v>
-      </c>
-      <c r="E140" s="25" t="n"/>
-    </row>
-    <row r="141" ht="18" customHeight="1">
-      <c r="A141" s="27" t="inlineStr">
+      <c r="B141" s="25" t="n"/>
+      <c r="C141" s="25" t="n"/>
+      <c r="D141" s="26" t="n">
+        <v>196555</v>
+      </c>
+      <c r="E141" s="25" t="n"/>
+    </row>
+    <row r="142" ht="18" customHeight="1">
+      <c r="A142" s="27" t="inlineStr">
         <is>
           <t xml:space="preserve">  Gary's Cut — 10% of (charge − pass-throughs $34,850)</t>
         </is>
       </c>
-      <c r="B141" s="27" t="n"/>
-      <c r="C141" s="27" t="n"/>
-      <c r="D141" s="28" t="n">
-        <v>16030</v>
-      </c>
-      <c r="E141" s="27" t="n"/>
-    </row>
-    <row r="142" ht="18" customHeight="1">
-      <c r="A142" s="29" t="inlineStr">
+      <c r="B142" s="27" t="n"/>
+      <c r="C142" s="27" t="n"/>
+      <c r="D142" s="28" t="n">
+        <v>16170</v>
+      </c>
+      <c r="E142" s="27" t="n"/>
+    </row>
+    <row r="143" ht="18" customHeight="1">
+      <c r="A143" s="29" t="inlineStr">
         <is>
           <t xml:space="preserve">  Gross Margin (before Gary)</t>
         </is>
       </c>
-      <c r="B142" s="29" t="n"/>
-      <c r="C142" s="29" t="n"/>
-      <c r="D142" s="30" t="n">
-        <v>54401</v>
-      </c>
-      <c r="E142" s="29" t="n"/>
-    </row>
-    <row r="143" ht="18" customHeight="1">
-      <c r="A143" s="25" t="inlineStr">
+      <c r="B143" s="29" t="n"/>
+      <c r="C143" s="29" t="n"/>
+      <c r="D143" s="30" t="n">
+        <v>54801</v>
+      </c>
+      <c r="E143" s="29" t="n"/>
+    </row>
+    <row r="144" ht="18" customHeight="1">
+      <c r="A144" s="25" t="inlineStr">
         <is>
           <t xml:space="preserve">  Justin Net Take-Home (after Gary)</t>
         </is>
       </c>
-      <c r="B143" s="25" t="n"/>
-      <c r="C143" s="25" t="n"/>
-      <c r="D143" s="26" t="n">
-        <v>38371</v>
-      </c>
-      <c r="E143" s="25" t="n"/>
-    </row>
-    <row r="144" ht="18" customHeight="1"/>
-    <row r="145">
-      <c r="A145" s="31" t="inlineStr">
+      <c r="B144" s="25" t="n"/>
+      <c r="C144" s="25" t="n"/>
+      <c r="D144" s="26" t="n">
+        <v>38631</v>
+      </c>
+      <c r="E144" s="25" t="n"/>
+    </row>
+    <row r="145"/>
+    <row r="146" ht="20" customHeight="1">
+      <c r="A146" s="31" t="inlineStr">
         <is>
           <t xml:space="preserve">  ✦  OPTIONAL ADD-ON — KITCHEN (Recommended — Not in Total)</t>
         </is>
       </c>
-      <c r="B145" s="31" t="n"/>
-      <c r="C145" s="31" t="n"/>
-      <c r="D145" s="31" t="n"/>
-      <c r="E145" s="31" t="n"/>
-    </row>
-    <row r="146" ht="20" customHeight="1">
-      <c r="A146" s="10" t="inlineStr">
+      <c r="B146" s="31" t="n"/>
+      <c r="C146" s="31" t="n"/>
+      <c r="D146" s="31" t="n"/>
+      <c r="E146" s="31" t="n"/>
+    </row>
+    <row r="147" ht="16" customHeight="1">
+      <c r="A147" s="10" t="inlineStr">
         <is>
           <t xml:space="preserve">  Demo existing kitchen (cabinets, counters, appliances)</t>
         </is>
       </c>
-      <c r="B146" s="11" t="n">
+      <c r="B147" s="11" t="n">
         <v>2000</v>
       </c>
-      <c r="C146" s="12" t="inlineStr">
-        <is>
-          <t>40%</t>
-        </is>
-      </c>
-      <c r="D146" s="11" t="n">
+      <c r="C147" s="12" t="inlineStr">
+        <is>
+          <t>40%</t>
+        </is>
+      </c>
+      <c r="D147" s="11" t="n">
         <v>2800</v>
       </c>
-      <c r="E146" s="13" t="inlineStr"/>
-    </row>
-    <row r="147" ht="16" customHeight="1">
-      <c r="A147" s="6" t="inlineStr">
+      <c r="E147" s="13" t="inlineStr"/>
+    </row>
+    <row r="148" ht="16" customHeight="1">
+      <c r="A148" s="6" t="inlineStr">
         <is>
           <t xml:space="preserve">  New cabinets — shaker style, standard allowance</t>
         </is>
       </c>
-      <c r="B147" s="7" t="n">
+      <c r="B148" s="7" t="n">
         <v>12000</v>
       </c>
-      <c r="C147" s="14" t="inlineStr">
-        <is>
-          <t>40%</t>
-        </is>
-      </c>
-      <c r="D147" s="7" t="n">
+      <c r="C148" s="14" t="inlineStr">
+        <is>
+          <t>40%</t>
+        </is>
+      </c>
+      <c r="D148" s="7" t="n">
         <v>16800</v>
       </c>
-      <c r="E147" s="9" t="inlineStr"/>
-    </row>
-    <row r="148" ht="16" customHeight="1">
-      <c r="A148" s="10" t="inlineStr">
+      <c r="E148" s="9" t="inlineStr"/>
+    </row>
+    <row r="149" ht="16" customHeight="1">
+      <c r="A149" s="10" t="inlineStr">
         <is>
           <t xml:space="preserve">  Cabinet installation labor (Don)</t>
         </is>
       </c>
-      <c r="B148" s="11" t="n">
+      <c r="B149" s="11" t="n">
         <v>3500</v>
       </c>
-      <c r="C148" s="12" t="inlineStr">
-        <is>
-          <t>40%</t>
-        </is>
-      </c>
-      <c r="D148" s="11" t="n">
+      <c r="C149" s="12" t="inlineStr">
+        <is>
+          <t>40%</t>
+        </is>
+      </c>
+      <c r="D149" s="11" t="n">
         <v>4900</v>
       </c>
-      <c r="E148" s="13" t="inlineStr"/>
-    </row>
-    <row r="149" ht="16" customHeight="1">
-      <c r="A149" s="6" t="inlineStr">
+      <c r="E149" s="13" t="inlineStr"/>
+    </row>
+    <row r="150" ht="16" customHeight="1">
+      <c r="A150" s="6" t="inlineStr">
         <is>
           <t xml:space="preserve">  Countertops — quartz allowance</t>
         </is>
       </c>
-      <c r="B149" s="7" t="n">
+      <c r="B150" s="7" t="n">
         <v>5000</v>
       </c>
-      <c r="C149" s="14" t="inlineStr">
-        <is>
-          <t>40%</t>
-        </is>
-      </c>
-      <c r="D149" s="7" t="n">
+      <c r="C150" s="14" t="inlineStr">
+        <is>
+          <t>40%</t>
+        </is>
+      </c>
+      <c r="D150" s="7" t="n">
         <v>7000</v>
       </c>
-      <c r="E149" s="9" t="inlineStr"/>
-    </row>
-    <row r="150" ht="16" customHeight="1">
-      <c r="A150" s="10" t="inlineStr">
+      <c r="E150" s="9" t="inlineStr"/>
+    </row>
+    <row r="151" ht="16" customHeight="1">
+      <c r="A151" s="10" t="inlineStr">
         <is>
           <t xml:space="preserve">  Backsplash tile — allowance</t>
         </is>
       </c>
-      <c r="B150" s="11" t="n">
+      <c r="B151" s="11" t="n">
         <v>1200</v>
       </c>
-      <c r="C150" s="12" t="inlineStr">
-        <is>
-          <t>40%</t>
-        </is>
-      </c>
-      <c r="D150" s="11" t="n">
+      <c r="C151" s="12" t="inlineStr">
+        <is>
+          <t>40%</t>
+        </is>
+      </c>
+      <c r="D151" s="11" t="n">
         <v>1680</v>
       </c>
-      <c r="E150" s="13" t="inlineStr"/>
-    </row>
-    <row r="151" ht="16" customHeight="1">
-      <c r="A151" s="6" t="inlineStr">
+      <c r="E151" s="13" t="inlineStr"/>
+    </row>
+    <row r="152" ht="16" customHeight="1">
+      <c r="A152" s="6" t="inlineStr">
         <is>
           <t xml:space="preserve">  Appliances — range, hood, dishwasher, fridge allowance</t>
         </is>
       </c>
-      <c r="B151" s="7" t="n">
+      <c r="B152" s="7" t="n">
         <v>6000</v>
       </c>
-      <c r="C151" s="14" t="inlineStr">
-        <is>
-          <t>40%</t>
-        </is>
-      </c>
-      <c r="D151" s="7" t="n">
+      <c r="C152" s="14" t="inlineStr">
+        <is>
+          <t>40%</t>
+        </is>
+      </c>
+      <c r="D152" s="7" t="n">
         <v>8400</v>
       </c>
-      <c r="E151" s="9" t="inlineStr"/>
-    </row>
-    <row r="152" ht="16" customHeight="1">
-      <c r="A152" s="10" t="inlineStr">
+      <c r="E152" s="9" t="inlineStr"/>
+    </row>
+    <row r="153" ht="16" customHeight="1">
+      <c r="A153" s="10" t="inlineStr">
         <is>
           <t xml:space="preserve">  Appliance installation</t>
         </is>
       </c>
-      <c r="B152" s="11" t="n">
+      <c r="B153" s="11" t="n">
         <v>1200</v>
       </c>
-      <c r="C152" s="12" t="inlineStr">
-        <is>
-          <t>40%</t>
-        </is>
-      </c>
-      <c r="D152" s="11" t="n">
+      <c r="C153" s="12" t="inlineStr">
+        <is>
+          <t>40%</t>
+        </is>
+      </c>
+      <c r="D153" s="11" t="n">
         <v>1680</v>
       </c>
-      <c r="E152" s="13" t="inlineStr"/>
-    </row>
-    <row r="153" ht="16" customHeight="1">
-      <c r="A153" s="6" t="inlineStr">
+      <c r="E153" s="13" t="inlineStr"/>
+    </row>
+    <row r="154" ht="16" customHeight="1">
+      <c r="A154" s="6" t="inlineStr">
         <is>
           <t xml:space="preserve">  Plumbing — sink/connection</t>
         </is>
       </c>
-      <c r="B153" s="7" t="n">
+      <c r="B154" s="7" t="n">
         <v>1000</v>
       </c>
-      <c r="C153" s="14" t="inlineStr">
-        <is>
-          <t>40%</t>
-        </is>
-      </c>
-      <c r="D153" s="7" t="n">
+      <c r="C154" s="14" t="inlineStr">
+        <is>
+          <t>40%</t>
+        </is>
+      </c>
+      <c r="D154" s="7" t="n">
         <v>1400</v>
       </c>
-      <c r="E153" s="9" t="inlineStr"/>
-    </row>
-    <row r="154" ht="16" customHeight="1">
-      <c r="A154" s="10" t="inlineStr">
+      <c r="E154" s="9" t="inlineStr"/>
+    </row>
+    <row r="155" ht="16" customHeight="1">
+      <c r="A155" s="10" t="inlineStr">
         <is>
           <t xml:space="preserve">  Electrical — dedicated circuits</t>
         </is>
       </c>
-      <c r="B154" s="11" t="n">
+      <c r="B155" s="11" t="n">
         <v>800</v>
       </c>
-      <c r="C154" s="12" t="inlineStr">
-        <is>
-          <t>40%</t>
-        </is>
-      </c>
-      <c r="D154" s="11" t="n">
+      <c r="C155" s="12" t="inlineStr">
+        <is>
+          <t>40%</t>
+        </is>
+      </c>
+      <c r="D155" s="11" t="n">
         <v>1120</v>
       </c>
-      <c r="E154" s="13" t="inlineStr"/>
-    </row>
-    <row r="155" ht="16" customHeight="1">
-      <c r="A155" s="32" t="inlineStr">
+      <c r="E155" s="13" t="inlineStr"/>
+    </row>
+    <row r="156" ht="20" customHeight="1">
+      <c r="A156" s="32" t="inlineStr">
         <is>
           <t xml:space="preserve">  ✦  OPTIONAL KITCHEN TOTAL</t>
         </is>
       </c>
-      <c r="B155" s="33" t="n">
+      <c r="B156" s="33" t="n">
         <v>32700</v>
       </c>
-      <c r="C155" s="32" t="n"/>
-      <c r="D155" s="33" t="n">
+      <c r="C156" s="32" t="n"/>
+      <c r="D156" s="33" t="n">
         <v>45780</v>
       </c>
-      <c r="E155" s="34" t="inlineStr">
+      <c r="E156" s="34" t="inlineStr">
         <is>
           <t>Add to contract if approved</t>
         </is>
       </c>
     </row>
-    <row r="156" ht="20" customHeight="1"/>
-    <row r="157">
-      <c r="A157" s="35" t="inlineStr">
+    <row r="157"/>
+    <row r="158" ht="22" customHeight="1">
+      <c r="A158" s="35" t="inlineStr">
         <is>
           <t xml:space="preserve">  ★★  TOTAL IF KITCHEN APPROVED</t>
         </is>
       </c>
-      <c r="B157" s="36" t="n">
-        <v>173454</v>
-      </c>
-      <c r="C157" s="35" t="n"/>
-      <c r="D157" s="36" t="n">
-        <v>240935</v>
-      </c>
-      <c r="E157" s="35" t="n"/>
-    </row>
-    <row r="158" ht="22" customHeight="1"/>
-    <row r="159">
-      <c r="A159" s="37" t="inlineStr">
+      <c r="B158" s="36" t="n">
+        <v>174454</v>
+      </c>
+      <c r="C158" s="35" t="n"/>
+      <c r="D158" s="36" t="n">
+        <v>242335</v>
+      </c>
+      <c r="E158" s="35" t="n"/>
+    </row>
+    <row r="159"/>
+    <row r="160" ht="18" customHeight="1">
+      <c r="A160" s="37" t="inlineStr">
         <is>
           <t xml:space="preserve">  NOTES &amp; ASSUMPTIONS</t>
         </is>
       </c>
-      <c r="B159" s="37" t="n"/>
-      <c r="C159" s="37" t="n"/>
-      <c r="D159" s="37" t="n"/>
-      <c r="E159" s="37" t="n"/>
-    </row>
-    <row r="160" ht="18" customHeight="1">
-      <c r="A160" s="38" t="inlineStr">
-        <is>
-          <t>• Window count (18) and sliding door count (2) are estimates — verify at site visit before ordering</t>
-        </is>
-      </c>
-      <c r="B160" s="39" t="n"/>
-      <c r="C160" s="39" t="n"/>
-      <c r="D160" s="39" t="n"/>
-      <c r="E160" s="39" t="n"/>
+      <c r="B160" s="37" t="n"/>
+      <c r="C160" s="37" t="n"/>
+      <c r="D160" s="37" t="n"/>
+      <c r="E160" s="37" t="n"/>
     </row>
     <row r="161" ht="15" customHeight="1">
       <c r="A161" s="38" t="inlineStr">
         <is>
-          <t>• LVP flooring ~1,900 SF excludes 7 bedrooms (~770 SF est.) and downstairs hallway per owner direction</t>
+          <t>• Window count (18) and sliding door count (2) are estimates — verify at site visit before ordering</t>
         </is>
       </c>
       <c r="B161" s="39" t="n"/>
@@ -3363,7 +3375,7 @@
     <row r="162" ht="15" customHeight="1">
       <c r="A162" s="38" t="inlineStr">
         <is>
-          <t>• Flooring subfloor prep / leveling NOT included — assess separately at site visit</t>
+          <t>• LVP flooring ~1,900 SF excludes 7 bedrooms (~770 SF est.) and downstairs hallway per owner direction</t>
         </is>
       </c>
       <c r="B162" s="39" t="n"/>
@@ -3374,7 +3386,7 @@
     <row r="163" ht="15" customHeight="1">
       <c r="A163" s="38" t="inlineStr">
         <is>
-          <t>• Main drain line repair is TBD pending video camera — budget as Change Order on discovery</t>
+          <t>• Flooring subfloor prep / leveling NOT included — assess separately at site visit</t>
         </is>
       </c>
       <c r="B163" s="39" t="n"/>
@@ -3385,7 +3397,7 @@
     <row r="164" ht="15" customHeight="1">
       <c r="A164" s="38" t="inlineStr">
         <is>
-          <t>• Mold remediation is a minimum estimate — full scope depends on IEP / environmental test report</t>
+          <t>• Main drain line repair is TBD pending video camera — budget as Change Order on discovery</t>
         </is>
       </c>
       <c r="B164" s="39" t="n"/>
@@ -3396,7 +3408,7 @@
     <row r="165" ht="15" customHeight="1">
       <c r="A165" s="38" t="inlineStr">
         <is>
-          <t>• All material allowances (tile, vanity, countertops, LVP, fixtures, appliances) are subject to client selections</t>
+          <t>• Mold remediation is a minimum estimate — full scope depends on IEP / environmental test report</t>
         </is>
       </c>
       <c r="B165" s="39" t="n"/>
@@ -3407,7 +3419,7 @@
     <row r="166" ht="15" customHeight="1">
       <c r="A166" s="38" t="inlineStr">
         <is>
-          <t>• Permit fees are estimated — final costs vary by Buena Park building dept. and scope</t>
+          <t>• All material allowances (tile, vanity, countertops, LVP, fixtures, appliances) are subject to client selections</t>
         </is>
       </c>
       <c r="B166" s="39" t="n"/>
@@ -3418,7 +3430,7 @@
     <row r="167" ht="15" customHeight="1">
       <c r="A167" s="38" t="inlineStr">
         <is>
-          <t>• Payment terms: 30% deposit / 40% at midpoint / 30% completion</t>
+          <t>• Permit fees are estimated — final costs vary by Buena Park building dept. and scope</t>
         </is>
       </c>
       <c r="B167" s="39" t="n"/>
@@ -3429,7 +3441,7 @@
     <row r="168" ht="15" customHeight="1">
       <c r="A168" s="38" t="inlineStr">
         <is>
-          <t>• Change orders require signed written approval before work proceeds</t>
+          <t>• Payment terms: 30% deposit / 40% at midpoint / 30% completion</t>
         </is>
       </c>
       <c r="B168" s="39" t="n"/>
@@ -3440,7 +3452,7 @@
     <row r="169" ht="15" customHeight="1">
       <c r="A169" s="38" t="inlineStr">
         <is>
-          <t>• Warranty: 1-year labor warranty; manufacturer warranties apply to all materials/fixtures</t>
+          <t>• Change orders require signed written approval before work proceeds</t>
         </is>
       </c>
       <c r="B169" s="39" t="n"/>
@@ -3451,7 +3463,7 @@
     <row r="170" ht="15" customHeight="1">
       <c r="A170" s="38" t="inlineStr">
         <is>
-          <t>• This budget is confidential — client-facing documents show total price only (no cost/margin)</t>
+          <t>• Warranty: 1-year labor warranty; manufacturer warranties apply to all materials/fixtures</t>
         </is>
       </c>
       <c r="B170" s="39" t="n"/>
@@ -3459,7 +3471,17 @@
       <c r="D170" s="39" t="n"/>
       <c r="E170" s="39" t="n"/>
     </row>
-    <row r="171" ht="15" customHeight="1"/>
+    <row r="171" ht="15" customHeight="1">
+      <c r="A171" s="38" t="inlineStr">
+        <is>
+          <t>• This budget is confidential — client-facing documents show total price only (no cost/margin)</t>
+        </is>
+      </c>
+      <c r="B171" s="39" t="n"/>
+      <c r="C171" s="39" t="n"/>
+      <c r="D171" s="39" t="n"/>
+      <c r="E171" s="39" t="n"/>
+    </row>
   </sheetData>
   <mergeCells count="16">
     <mergeCell ref="A114:E114"/>

</xml_diff>

<commit_message>
Rebuild kitchen budget per Justin: new pricing, pass-throughs, drop appliances
</commit_message>
<xml_diff>
--- a/docs/san-palo-circle-robert-bird/San-Palo-Circle-Budget.xlsx
+++ b/docs/san-palo-circle-robert-bird/San-Palo-Circle-Budget.xlsx
@@ -730,7 +730,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E171"/>
+  <dimension ref="A1:E170"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -905,10 +905,10 @@
     </row>
     <row r="11" ht="18" customHeight="1">
       <c r="A11" s="17" t="n"/>
-      <c r="B11" s="17" t="n"/>
-      <c r="C11" s="17" t="n"/>
-      <c r="D11" s="17" t="n"/>
-      <c r="E11" s="17" t="n"/>
+      <c r="B11" s="40" t="n"/>
+      <c r="C11" s="40" t="n"/>
+      <c r="D11" s="40" t="n"/>
+      <c r="E11" s="41" t="n"/>
     </row>
     <row r="12" ht="16" customHeight="1">
       <c r="A12" s="4" t="inlineStr">
@@ -1208,10 +1208,10 @@
     </row>
     <row r="28" ht="18" customHeight="1">
       <c r="A28" s="17" t="n"/>
-      <c r="B28" s="17" t="n"/>
-      <c r="C28" s="17" t="n"/>
-      <c r="D28" s="17" t="n"/>
-      <c r="E28" s="17" t="n"/>
+      <c r="B28" s="40" t="n"/>
+      <c r="C28" s="40" t="n"/>
+      <c r="D28" s="40" t="n"/>
+      <c r="E28" s="41" t="n"/>
     </row>
     <row r="29" ht="16" customHeight="1">
       <c r="A29" s="4" t="inlineStr">
@@ -1507,10 +1507,10 @@
     </row>
     <row r="45" ht="18" customHeight="1">
       <c r="A45" s="17" t="n"/>
-      <c r="B45" s="17" t="n"/>
-      <c r="C45" s="17" t="n"/>
-      <c r="D45" s="17" t="n"/>
-      <c r="E45" s="17" t="n"/>
+      <c r="B45" s="40" t="n"/>
+      <c r="C45" s="40" t="n"/>
+      <c r="D45" s="40" t="n"/>
+      <c r="E45" s="41" t="n"/>
     </row>
     <row r="46" ht="16" customHeight="1">
       <c r="A46" s="4" t="inlineStr">
@@ -1806,10 +1806,10 @@
     </row>
     <row r="62" ht="18" customHeight="1">
       <c r="A62" s="17" t="n"/>
-      <c r="B62" s="17" t="n"/>
-      <c r="C62" s="17" t="n"/>
-      <c r="D62" s="17" t="n"/>
-      <c r="E62" s="17" t="n"/>
+      <c r="B62" s="40" t="n"/>
+      <c r="C62" s="40" t="n"/>
+      <c r="D62" s="40" t="n"/>
+      <c r="E62" s="41" t="n"/>
     </row>
     <row r="63" ht="16" customHeight="1">
       <c r="A63" s="4" t="inlineStr">
@@ -1976,10 +1976,10 @@
     </row>
     <row r="72" ht="18" customHeight="1">
       <c r="A72" s="17" t="n"/>
-      <c r="B72" s="17" t="n"/>
-      <c r="C72" s="17" t="n"/>
-      <c r="D72" s="17" t="n"/>
-      <c r="E72" s="17" t="n"/>
+      <c r="B72" s="40" t="n"/>
+      <c r="C72" s="40" t="n"/>
+      <c r="D72" s="40" t="n"/>
+      <c r="E72" s="41" t="n"/>
     </row>
     <row r="73" ht="16" customHeight="1">
       <c r="A73" s="4" t="inlineStr">
@@ -2093,10 +2093,10 @@
     </row>
     <row r="79" ht="18" customHeight="1">
       <c r="A79" s="17" t="n"/>
-      <c r="B79" s="17" t="n"/>
-      <c r="C79" s="17" t="n"/>
-      <c r="D79" s="17" t="n"/>
-      <c r="E79" s="17" t="n"/>
+      <c r="B79" s="40" t="n"/>
+      <c r="C79" s="40" t="n"/>
+      <c r="D79" s="40" t="n"/>
+      <c r="E79" s="41" t="n"/>
     </row>
     <row r="80" ht="16" customHeight="1">
       <c r="A80" s="4" t="inlineStr">
@@ -2210,10 +2210,10 @@
     </row>
     <row r="86" ht="18" customHeight="1">
       <c r="A86" s="17" t="n"/>
-      <c r="B86" s="17" t="n"/>
-      <c r="C86" s="17" t="n"/>
-      <c r="D86" s="17" t="n"/>
-      <c r="E86" s="17" t="n"/>
+      <c r="B86" s="40" t="n"/>
+      <c r="C86" s="40" t="n"/>
+      <c r="D86" s="40" t="n"/>
+      <c r="E86" s="41" t="n"/>
     </row>
     <row r="87" ht="16" customHeight="1">
       <c r="A87" s="4" t="inlineStr">
@@ -2369,10 +2369,10 @@
     </row>
     <row r="95" ht="18" customHeight="1">
       <c r="A95" s="17" t="n"/>
-      <c r="B95" s="17" t="n"/>
-      <c r="C95" s="17" t="n"/>
-      <c r="D95" s="17" t="n"/>
-      <c r="E95" s="17" t="n"/>
+      <c r="B95" s="40" t="n"/>
+      <c r="C95" s="40" t="n"/>
+      <c r="D95" s="40" t="n"/>
+      <c r="E95" s="41" t="n"/>
     </row>
     <row r="96" ht="16" customHeight="1">
       <c r="A96" s="4" t="inlineStr">
@@ -2463,10 +2463,10 @@
     </row>
     <row r="101" ht="18" customHeight="1">
       <c r="A101" s="17" t="n"/>
-      <c r="B101" s="17" t="n"/>
-      <c r="C101" s="17" t="n"/>
-      <c r="D101" s="17" t="n"/>
-      <c r="E101" s="17" t="n"/>
+      <c r="B101" s="40" t="n"/>
+      <c r="C101" s="40" t="n"/>
+      <c r="D101" s="40" t="n"/>
+      <c r="E101" s="41" t="n"/>
     </row>
     <row r="102" ht="16" customHeight="1">
       <c r="A102" s="4" t="inlineStr">
@@ -2572,10 +2572,10 @@
     </row>
     <row r="108" ht="18" customHeight="1">
       <c r="A108" s="17" t="n"/>
-      <c r="B108" s="17" t="n"/>
-      <c r="C108" s="17" t="n"/>
-      <c r="D108" s="17" t="n"/>
-      <c r="E108" s="17" t="n"/>
+      <c r="B108" s="40" t="n"/>
+      <c r="C108" s="40" t="n"/>
+      <c r="D108" s="40" t="n"/>
+      <c r="E108" s="41" t="n"/>
     </row>
     <row r="109" ht="16" customHeight="1">
       <c r="A109" s="4" t="inlineStr">
@@ -2662,10 +2662,10 @@
     </row>
     <row r="114" ht="18" customHeight="1">
       <c r="A114" s="17" t="n"/>
-      <c r="B114" s="17" t="n"/>
-      <c r="C114" s="17" t="n"/>
-      <c r="D114" s="17" t="n"/>
-      <c r="E114" s="17" t="n"/>
+      <c r="B114" s="40" t="n"/>
+      <c r="C114" s="40" t="n"/>
+      <c r="D114" s="40" t="n"/>
+      <c r="E114" s="41" t="n"/>
     </row>
     <row r="115" ht="16" customHeight="1">
       <c r="A115" s="4" t="inlineStr">
@@ -2771,10 +2771,10 @@
     </row>
     <row r="121" ht="18" customHeight="1">
       <c r="A121" s="17" t="n"/>
-      <c r="B121" s="17" t="n"/>
-      <c r="C121" s="17" t="n"/>
-      <c r="D121" s="17" t="n"/>
-      <c r="E121" s="17" t="n"/>
+      <c r="B121" s="40" t="n"/>
+      <c r="C121" s="40" t="n"/>
+      <c r="D121" s="40" t="n"/>
+      <c r="E121" s="41" t="n"/>
     </row>
     <row r="122" ht="16" customHeight="1">
       <c r="A122" s="4" t="inlineStr">
@@ -2945,10 +2945,10 @@
     </row>
     <row r="131" ht="18" customHeight="1">
       <c r="A131" s="17" t="n"/>
-      <c r="B131" s="17" t="n"/>
-      <c r="C131" s="17" t="n"/>
-      <c r="D131" s="17" t="n"/>
-      <c r="E131" s="17" t="n"/>
+      <c r="B131" s="40" t="n"/>
+      <c r="C131" s="40" t="n"/>
+      <c r="D131" s="40" t="n"/>
+      <c r="E131" s="41" t="n"/>
     </row>
     <row r="132" ht="16" customHeight="1">
       <c r="A132" s="4" t="inlineStr">
@@ -3078,7 +3078,6 @@
         </is>
       </c>
     </row>
-    <row r="140"/>
     <row r="141" ht="18" customHeight="1">
       <c r="A141" s="25" t="inlineStr">
         <is>
@@ -3131,7 +3130,6 @@
       </c>
       <c r="E144" s="25" t="n"/>
     </row>
-    <row r="145"/>
     <row r="146" ht="20" customHeight="1">
       <c r="A146" s="31" t="inlineStr">
         <is>
@@ -3146,11 +3144,11 @@
     <row r="147" ht="16" customHeight="1">
       <c r="A147" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Demo existing kitchen (cabinets, counters, appliances)</t>
+          <t xml:space="preserve">  Demo existing kitchen (cabinets, counters, tile)</t>
         </is>
       </c>
       <c r="B147" s="11" t="n">
-        <v>2000</v>
+        <v>1400</v>
       </c>
       <c r="C147" s="12" t="inlineStr">
         <is>
@@ -3158,37 +3156,41 @@
         </is>
       </c>
       <c r="D147" s="11" t="n">
-        <v>2800</v>
-      </c>
-      <c r="E147" s="13" t="inlineStr"/>
+        <v>1960</v>
+      </c>
+      <c r="E147" s="13" t="n"/>
     </row>
     <row r="148" ht="16" customHeight="1">
       <c r="A148" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">  New cabinets — shaker style, standard allowance</t>
+          <t xml:space="preserve">  Cabinet material — allowance (pass-through)</t>
         </is>
       </c>
       <c r="B148" s="7" t="n">
-        <v>12000</v>
+        <v>10000</v>
       </c>
       <c r="C148" s="14" t="inlineStr">
         <is>
-          <t>40%</t>
+          <t>pass-through</t>
         </is>
       </c>
       <c r="D148" s="7" t="n">
-        <v>16800</v>
-      </c>
-      <c r="E148" s="9" t="inlineStr"/>
+        <v>10000</v>
+      </c>
+      <c r="E148" s="9" t="inlineStr">
+        <is>
+          <t>Client-selected; at cost</t>
+        </is>
+      </c>
     </row>
     <row r="149" ht="16" customHeight="1">
       <c r="A149" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Cabinet installation labor (Don)</t>
+          <t xml:space="preserve">  Cabinet installation labor</t>
         </is>
       </c>
       <c r="B149" s="11" t="n">
-        <v>3500</v>
+        <v>2857</v>
       </c>
       <c r="C149" s="12" t="inlineStr">
         <is>
@@ -3196,56 +3198,64 @@
         </is>
       </c>
       <c r="D149" s="11" t="n">
-        <v>4900</v>
-      </c>
-      <c r="E149" s="13" t="inlineStr"/>
+        <v>4000</v>
+      </c>
+      <c r="E149" s="13" t="n"/>
     </row>
     <row r="150" ht="16" customHeight="1">
       <c r="A150" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Countertops — quartz allowance</t>
+          <t xml:space="preserve">  Countertops — allowance (pass-through)</t>
         </is>
       </c>
       <c r="B150" s="7" t="n">
-        <v>5000</v>
+        <v>7000</v>
       </c>
       <c r="C150" s="14" t="inlineStr">
         <is>
-          <t>40%</t>
+          <t>pass-through</t>
         </is>
       </c>
       <c r="D150" s="7" t="n">
         <v>7000</v>
       </c>
-      <c r="E150" s="9" t="inlineStr"/>
+      <c r="E150" s="9" t="inlineStr">
+        <is>
+          <t>Client-selected; at cost</t>
+        </is>
+      </c>
     </row>
     <row r="151" ht="16" customHeight="1">
       <c r="A151" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Backsplash tile — allowance</t>
+          <t xml:space="preserve">  Backsplash tile material — allowance (pass-through)</t>
         </is>
       </c>
       <c r="B151" s="11" t="n">
-        <v>1200</v>
+        <v>800</v>
       </c>
       <c r="C151" s="12" t="inlineStr">
         <is>
-          <t>40%</t>
+          <t>pass-through</t>
         </is>
       </c>
       <c r="D151" s="11" t="n">
-        <v>1680</v>
-      </c>
-      <c r="E151" s="13" t="inlineStr"/>
+        <v>800</v>
+      </c>
+      <c r="E151" s="13" t="inlineStr">
+        <is>
+          <t>Client-selected; at cost</t>
+        </is>
+      </c>
     </row>
     <row r="152" ht="16" customHeight="1">
       <c r="A152" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Appliances — range, hood, dishwasher, fridge allowance</t>
+          <t xml:space="preserve">  Backsplash tile labor</t>
         </is>
       </c>
       <c r="B152" s="7" t="n">
-        <v>6000</v>
+        <v>571</v>
       </c>
       <c r="C152" s="14" t="inlineStr">
         <is>
@@ -3253,18 +3263,18 @@
         </is>
       </c>
       <c r="D152" s="7" t="n">
-        <v>8400</v>
-      </c>
-      <c r="E152" s="9" t="inlineStr"/>
+        <v>800</v>
+      </c>
+      <c r="E152" s="9" t="n"/>
     </row>
     <row r="153" ht="16" customHeight="1">
       <c r="A153" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Appliance installation</t>
+          <t xml:space="preserve">  Plumbing — sink/connection</t>
         </is>
       </c>
       <c r="B153" s="11" t="n">
-        <v>1200</v>
+        <v>571</v>
       </c>
       <c r="C153" s="12" t="inlineStr">
         <is>
@@ -3272,18 +3282,18 @@
         </is>
       </c>
       <c r="D153" s="11" t="n">
-        <v>1680</v>
-      </c>
-      <c r="E153" s="13" t="inlineStr"/>
+        <v>800</v>
+      </c>
+      <c r="E153" s="13" t="n"/>
     </row>
     <row r="154" ht="16" customHeight="1">
       <c r="A154" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Plumbing — sink/connection</t>
+          <t xml:space="preserve">  Electrical — dedicated circuits</t>
         </is>
       </c>
       <c r="B154" s="7" t="n">
-        <v>1000</v>
+        <v>429</v>
       </c>
       <c r="C154" s="14" t="inlineStr">
         <is>
@@ -3291,80 +3301,72 @@
         </is>
       </c>
       <c r="D154" s="7" t="n">
-        <v>1400</v>
-      </c>
-      <c r="E154" s="9" t="inlineStr"/>
+        <v>600</v>
+      </c>
+      <c r="E154" s="9" t="n"/>
     </row>
     <row r="155" ht="16" customHeight="1">
-      <c r="A155" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Electrical — dedicated circuits</t>
-        </is>
-      </c>
-      <c r="B155" s="11" t="n">
-        <v>800</v>
-      </c>
-      <c r="C155" s="12" t="inlineStr">
-        <is>
-          <t>40%</t>
-        </is>
-      </c>
-      <c r="D155" s="11" t="n">
-        <v>1120</v>
-      </c>
-      <c r="E155" s="13" t="inlineStr"/>
-    </row>
-    <row r="156" ht="20" customHeight="1">
-      <c r="A156" s="32" t="inlineStr">
+      <c r="A155" s="32" t="inlineStr">
         <is>
           <t xml:space="preserve">  ✦  OPTIONAL KITCHEN TOTAL</t>
         </is>
       </c>
-      <c r="B156" s="33" t="n">
-        <v>32700</v>
-      </c>
-      <c r="C156" s="32" t="n"/>
-      <c r="D156" s="33" t="n">
-        <v>45780</v>
-      </c>
-      <c r="E156" s="34" t="inlineStr">
+      <c r="B155" s="33" t="n">
+        <v>23628</v>
+      </c>
+      <c r="C155" s="32" t="n"/>
+      <c r="D155" s="33" t="n">
+        <v>25960</v>
+      </c>
+      <c r="E155" s="34" t="inlineStr">
         <is>
           <t>Add to contract if approved</t>
         </is>
       </c>
     </row>
-    <row r="157"/>
-    <row r="158" ht="22" customHeight="1">
-      <c r="A158" s="35" t="inlineStr">
+    <row r="156" ht="20" customHeight="1"/>
+    <row r="157">
+      <c r="A157" s="35" t="inlineStr">
         <is>
           <t xml:space="preserve">  ★★  TOTAL IF KITCHEN APPROVED</t>
         </is>
       </c>
-      <c r="B158" s="36" t="n">
-        <v>174454</v>
-      </c>
-      <c r="C158" s="35" t="n"/>
-      <c r="D158" s="36" t="n">
-        <v>242335</v>
-      </c>
-      <c r="E158" s="35" t="n"/>
-    </row>
-    <row r="159"/>
+      <c r="B157" s="36" t="n">
+        <v>165382</v>
+      </c>
+      <c r="C157" s="35" t="n"/>
+      <c r="D157" s="36" t="n">
+        <v>222515</v>
+      </c>
+      <c r="E157" s="35" t="n"/>
+    </row>
+    <row r="158" ht="22" customHeight="1"/>
+    <row r="159">
+      <c r="A159" s="37" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  NOTES &amp; ASSUMPTIONS</t>
+        </is>
+      </c>
+      <c r="B159" s="37" t="n"/>
+      <c r="C159" s="37" t="n"/>
+      <c r="D159" s="37" t="n"/>
+      <c r="E159" s="37" t="n"/>
+    </row>
     <row r="160" ht="18" customHeight="1">
-      <c r="A160" s="37" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  NOTES &amp; ASSUMPTIONS</t>
-        </is>
-      </c>
-      <c r="B160" s="37" t="n"/>
-      <c r="C160" s="37" t="n"/>
-      <c r="D160" s="37" t="n"/>
-      <c r="E160" s="37" t="n"/>
+      <c r="A160" s="38" t="inlineStr">
+        <is>
+          <t>• Window count (18) and sliding door count (2) are estimates — verify at site visit before ordering</t>
+        </is>
+      </c>
+      <c r="B160" s="39" t="n"/>
+      <c r="C160" s="39" t="n"/>
+      <c r="D160" s="39" t="n"/>
+      <c r="E160" s="39" t="n"/>
     </row>
     <row r="161" ht="15" customHeight="1">
       <c r="A161" s="38" t="inlineStr">
         <is>
-          <t>• Window count (18) and sliding door count (2) are estimates — verify at site visit before ordering</t>
+          <t>• LVP flooring ~1,900 SF excludes 7 bedrooms (~770 SF est.) and downstairs hallway per owner direction</t>
         </is>
       </c>
       <c r="B161" s="39" t="n"/>
@@ -3375,7 +3377,7 @@
     <row r="162" ht="15" customHeight="1">
       <c r="A162" s="38" t="inlineStr">
         <is>
-          <t>• LVP flooring ~1,900 SF excludes 7 bedrooms (~770 SF est.) and downstairs hallway per owner direction</t>
+          <t>• Flooring subfloor prep / leveling NOT included — assess separately at site visit</t>
         </is>
       </c>
       <c r="B162" s="39" t="n"/>
@@ -3386,7 +3388,7 @@
     <row r="163" ht="15" customHeight="1">
       <c r="A163" s="38" t="inlineStr">
         <is>
-          <t>• Flooring subfloor prep / leveling NOT included — assess separately at site visit</t>
+          <t>• Main drain line repair is TBD pending video camera — budget as Change Order on discovery</t>
         </is>
       </c>
       <c r="B163" s="39" t="n"/>
@@ -3397,7 +3399,7 @@
     <row r="164" ht="15" customHeight="1">
       <c r="A164" s="38" t="inlineStr">
         <is>
-          <t>• Main drain line repair is TBD pending video camera — budget as Change Order on discovery</t>
+          <t>• Mold remediation is a minimum estimate — full scope depends on IEP / environmental test report</t>
         </is>
       </c>
       <c r="B164" s="39" t="n"/>
@@ -3408,7 +3410,7 @@
     <row r="165" ht="15" customHeight="1">
       <c r="A165" s="38" t="inlineStr">
         <is>
-          <t>• Mold remediation is a minimum estimate — full scope depends on IEP / environmental test report</t>
+          <t>• All material allowances (tile, vanity, countertops, LVP, fixtures, appliances) are subject to client selections</t>
         </is>
       </c>
       <c r="B165" s="39" t="n"/>
@@ -3419,7 +3421,7 @@
     <row r="166" ht="15" customHeight="1">
       <c r="A166" s="38" t="inlineStr">
         <is>
-          <t>• All material allowances (tile, vanity, countertops, LVP, fixtures, appliances) are subject to client selections</t>
+          <t>• Permit fees are estimated — final costs vary by Buena Park building dept. and scope</t>
         </is>
       </c>
       <c r="B166" s="39" t="n"/>
@@ -3430,7 +3432,7 @@
     <row r="167" ht="15" customHeight="1">
       <c r="A167" s="38" t="inlineStr">
         <is>
-          <t>• Permit fees are estimated — final costs vary by Buena Park building dept. and scope</t>
+          <t>• Payment terms: 30% deposit / 40% at midpoint / 30% completion</t>
         </is>
       </c>
       <c r="B167" s="39" t="n"/>
@@ -3441,7 +3443,7 @@
     <row r="168" ht="15" customHeight="1">
       <c r="A168" s="38" t="inlineStr">
         <is>
-          <t>• Payment terms: 30% deposit / 40% at midpoint / 30% completion</t>
+          <t>• Change orders require signed written approval before work proceeds</t>
         </is>
       </c>
       <c r="B168" s="39" t="n"/>
@@ -3452,7 +3454,7 @@
     <row r="169" ht="15" customHeight="1">
       <c r="A169" s="38" t="inlineStr">
         <is>
-          <t>• Change orders require signed written approval before work proceeds</t>
+          <t>• Warranty: 1-year labor warranty; manufacturer warranties apply to all materials/fixtures</t>
         </is>
       </c>
       <c r="B169" s="39" t="n"/>
@@ -3463,7 +3465,7 @@
     <row r="170" ht="15" customHeight="1">
       <c r="A170" s="38" t="inlineStr">
         <is>
-          <t>• Warranty: 1-year labor warranty; manufacturer warranties apply to all materials/fixtures</t>
+          <t>• This budget is confidential — client-facing documents show total price only (no cost/margin)</t>
         </is>
       </c>
       <c r="B170" s="39" t="n"/>
@@ -3471,17 +3473,7 @@
       <c r="D170" s="39" t="n"/>
       <c r="E170" s="39" t="n"/>
     </row>
-    <row r="171" ht="15" customHeight="1">
-      <c r="A171" s="38" t="inlineStr">
-        <is>
-          <t>• This budget is confidential — client-facing documents show total price only (no cost/margin)</t>
-        </is>
-      </c>
-      <c r="B171" s="39" t="n"/>
-      <c r="C171" s="39" t="n"/>
-      <c r="D171" s="39" t="n"/>
-      <c r="E171" s="39" t="n"/>
-    </row>
+    <row r="171" ht="15" customHeight="1"/>
   </sheetData>
   <mergeCells count="16">
     <mergeCell ref="A114:E114"/>

</xml_diff>

<commit_message>
Update proposal: ceiling/exterior/electrical/plumbing revisions per Justin, new totals $155,481
</commit_message>
<xml_diff>
--- a/docs/san-palo-circle-robert-bird/San-Palo-Circle-Budget.xlsx
+++ b/docs/san-palo-circle-robert-bird/San-Palo-Circle-Budget.xlsx
@@ -2022,11 +2022,7 @@
       <c r="E76" s="41" t="n"/>
     </row>
     <row r="77" ht="18" customHeight="1">
-      <c r="A77" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Asbestos pre-test — REQUIRED (pre-1980 home)</t>
-        </is>
-      </c>
+      <c r="A77" s="10" t="n"/>
       <c r="B77" s="40" t="n"/>
       <c r="C77" s="40" t="n"/>
       <c r="D77" s="40" t="n"/>
@@ -2035,93 +2031,45 @@
     <row r="78" ht="6" customHeight="1">
       <c r="A78" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Popcorn ceiling scrape — full house ~2,668 SF</t>
+          <t xml:space="preserve">  Popcorn ceiling scrape &amp; re-texture — full house</t>
         </is>
       </c>
       <c r="B78" s="7" t="n">
+        <v>2857</v>
+      </c>
+      <c r="C78" s="14" t="inlineStr">
+        <is>
+          <t>40%</t>
+        </is>
+      </c>
+      <c r="D78" s="7" t="n">
         <v>4000</v>
       </c>
-      <c r="C78" s="14" t="inlineStr">
-        <is>
-          <t>40%</t>
-        </is>
-      </c>
-      <c r="D78" s="7" t="n">
-        <v>5600</v>
-      </c>
-      <c r="E78" s="9" t="inlineStr">
-        <is>
-          <t>Wet scrape method</t>
-        </is>
-      </c>
+      <c r="E78" s="9" t="n"/>
     </row>
     <row r="79" ht="18" customHeight="1">
-      <c r="A79" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Remove &amp; replace existing fixtures (~15 units)</t>
-        </is>
-      </c>
+      <c r="A79" s="10" t="n"/>
     </row>
     <row r="80" ht="16" customHeight="1">
-      <c r="A80" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  New recessed can lights — ~25 added throughout</t>
-        </is>
-      </c>
-      <c r="B80" s="7" t="n">
-        <v>5000</v>
-      </c>
-      <c r="C80" s="14" t="inlineStr">
-        <is>
-          <t>40%</t>
-        </is>
-      </c>
-      <c r="D80" s="7" t="n">
-        <v>7000</v>
-      </c>
-      <c r="E80" s="9" t="inlineStr">
-        <is>
-          <t>Labor + fixtures incl.</t>
-        </is>
-      </c>
+      <c r="A80" s="6" t="n"/>
+      <c r="B80" s="7" t="n"/>
+      <c r="C80" s="14" t="n"/>
+      <c r="D80" s="7" t="n"/>
+      <c r="E80" s="9" t="n"/>
     </row>
     <row r="81" ht="16" customHeight="1">
-      <c r="A81" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Electrical — new circuits, switch boxes, dimmers</t>
-        </is>
-      </c>
-      <c r="B81" s="11" t="n">
-        <v>2000</v>
-      </c>
-      <c r="C81" s="12" t="inlineStr">
-        <is>
-          <t>40%</t>
-        </is>
-      </c>
-      <c r="D81" s="11" t="n">
-        <v>2800</v>
-      </c>
-      <c r="E81" s="13" t="inlineStr"/>
+      <c r="A81" s="10" t="n"/>
+      <c r="B81" s="11" t="n"/>
+      <c r="C81" s="12" t="n"/>
+      <c r="D81" s="11" t="n"/>
+      <c r="E81" s="13" t="n"/>
     </row>
     <row r="82" ht="16" customHeight="1">
-      <c r="A82" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Dimmer switches — select rooms</t>
-        </is>
-      </c>
-      <c r="B82" s="7" t="n">
-        <v>600</v>
-      </c>
-      <c r="C82" s="14" t="inlineStr">
-        <is>
-          <t>40%</t>
-        </is>
-      </c>
-      <c r="D82" s="7" t="n">
-        <v>840</v>
-      </c>
-      <c r="E82" s="9" t="inlineStr"/>
+      <c r="A82" s="6" t="n"/>
+      <c r="B82" s="7" t="n"/>
+      <c r="C82" s="14" t="n"/>
+      <c r="D82" s="7" t="n"/>
+      <c r="E82" s="9" t="n"/>
     </row>
     <row r="83" ht="16" customHeight="1">
       <c r="A83" s="15" t="inlineStr">
@@ -2130,11 +2078,11 @@
         </is>
       </c>
       <c r="B83" s="40" t="n">
-        <v>14100</v>
+        <v>2857</v>
       </c>
       <c r="C83" s="40" t="n"/>
       <c r="D83" s="40" t="n">
-        <v>19740</v>
+        <v>4000</v>
       </c>
       <c r="E83" s="41" t="n"/>
     </row>
@@ -2170,7 +2118,7 @@
         </is>
       </c>
       <c r="B87" s="11" t="n">
-        <v>1800</v>
+        <v>857</v>
       </c>
       <c r="C87" s="12" t="inlineStr">
         <is>
@@ -2178,28 +2126,16 @@
         </is>
       </c>
       <c r="D87" s="11" t="n">
-        <v>2520</v>
-      </c>
-      <c r="E87" s="13" t="inlineStr"/>
+        <v>1200</v>
+      </c>
+      <c r="E87" s="13" t="n"/>
     </row>
     <row r="88" ht="16" customHeight="1">
-      <c r="A88" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Deck stain &amp; weatherproofing</t>
-        </is>
-      </c>
-      <c r="B88" s="7" t="n">
-        <v>600</v>
-      </c>
-      <c r="C88" s="14" t="inlineStr">
-        <is>
-          <t>40%</t>
-        </is>
-      </c>
-      <c r="D88" s="7" t="n">
-        <v>840</v>
-      </c>
-      <c r="E88" s="9" t="inlineStr"/>
+      <c r="A88" s="6" t="n"/>
+      <c r="B88" s="7" t="n"/>
+      <c r="C88" s="14" t="n"/>
+      <c r="D88" s="7" t="n"/>
+      <c r="E88" s="9" t="n"/>
     </row>
     <row r="89" ht="16" customHeight="1">
       <c r="A89" s="15" t="inlineStr">
@@ -2208,11 +2144,11 @@
         </is>
       </c>
       <c r="B89" s="16" t="n">
-        <v>4900</v>
+        <v>857</v>
       </c>
       <c r="C89" s="15" t="n"/>
       <c r="D89" s="16" t="n">
-        <v>6860</v>
+        <v>1200</v>
       </c>
       <c r="E89" s="15" t="n"/>
     </row>
@@ -2414,7 +2350,7 @@
         </is>
       </c>
       <c r="B107" s="11" t="n">
-        <v>4500</v>
+        <v>4050</v>
       </c>
       <c r="C107" s="12" t="inlineStr">
         <is>
@@ -2422,7 +2358,7 @@
         </is>
       </c>
       <c r="D107" s="11" t="n">
-        <v>6300</v>
+        <v>5670</v>
       </c>
       <c r="E107" s="13" t="inlineStr"/>
     </row>
@@ -2440,11 +2376,11 @@
         </is>
       </c>
       <c r="B109" s="16" t="n">
-        <v>10100</v>
+        <v>9090</v>
       </c>
       <c r="C109" s="15" t="n"/>
       <c r="D109" s="16" t="n">
-        <v>14140</v>
+        <v>12726</v>
       </c>
       <c r="E109" s="15" t="n"/>
     </row>
@@ -2578,11 +2514,11 @@
         </is>
       </c>
       <c r="B119" s="40" t="n">
-        <v>7500</v>
+        <v>6071</v>
       </c>
       <c r="C119" s="40" t="n"/>
       <c r="D119" s="40" t="n">
-        <v>10500</v>
+        <v>8500</v>
       </c>
       <c r="E119" s="41" t="n"/>
     </row>
@@ -2705,11 +2641,11 @@
         </is>
       </c>
       <c r="B128" s="40" t="n">
-        <v>132111</v>
+        <v>114386</v>
       </c>
       <c r="C128" s="40" t="n"/>
       <c r="D128" s="40" t="n">
-        <v>180295</v>
+        <v>155481</v>
       </c>
       <c r="E128" s="41" t="n"/>
     </row>
@@ -2723,7 +2659,7 @@
       <c r="B130" s="25" t="n"/>
       <c r="C130" s="25" t="n"/>
       <c r="D130" s="26" t="n">
-        <v>180295</v>
+        <v>155481</v>
       </c>
       <c r="E130" s="25" t="n"/>
     </row>
@@ -2734,7 +2670,7 @@
         </is>
       </c>
       <c r="D131" t="n">
-        <v>16864</v>
+        <v>14383</v>
       </c>
     </row>
     <row r="132" ht="16" customHeight="1">
@@ -2746,7 +2682,7 @@
       <c r="B132" s="29" t="n"/>
       <c r="C132" s="29" t="n"/>
       <c r="D132" s="30" t="n">
-        <v>48184</v>
+        <v>41095</v>
       </c>
       <c r="E132" s="29" t="n"/>
     </row>
@@ -2759,7 +2695,7 @@
       <c r="B133" s="25" t="n"/>
       <c r="C133" s="25" t="n"/>
       <c r="D133" s="26" t="n">
-        <v>31320</v>
+        <v>26712</v>
       </c>
       <c r="E133" s="25" t="n"/>
     </row>
@@ -2966,11 +2902,11 @@
         </is>
       </c>
       <c r="B146" s="36" t="n">
-        <v>155739</v>
+        <v>138014</v>
       </c>
       <c r="C146" s="35" t="n"/>
       <c r="D146" s="36" t="n">
-        <v>206255</v>
+        <v>181441</v>
       </c>
       <c r="E146" s="35" t="n"/>
     </row>

</xml_diff>

<commit_message>
Flooring to 1,800 SF; iron railing $3,000; new project total $154,971
</commit_message>
<xml_diff>
--- a/docs/san-palo-circle-robert-bird/San-Palo-Circle-Budget.xlsx
+++ b/docs/san-palo-circle-robert-bird/San-Palo-Circle-Budget.xlsx
@@ -785,18 +785,18 @@
     <row r="5" ht="18" customHeight="1">
       <c r="A5" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">  01 — FLOORING (LVP — excludes bedrooms &amp; downstairs hallway | ~1,900 SF)</t>
+          <t xml:space="preserve">  01 — FLOORING (LVP — excludes 2 bedrooms &amp; downstairs hardwood hallway | ~1,800 SF)</t>
         </is>
       </c>
     </row>
     <row r="6" ht="16" customHeight="1">
       <c r="A6" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">  LVP material — 2,340 SF @ $2.50/SF allowance</t>
+          <t xml:space="preserve">  LVP material — 1800 SF @ $2.50/SF allowance</t>
         </is>
       </c>
       <c r="B6" s="7" t="n">
-        <v>5850</v>
+        <v>4500</v>
       </c>
       <c r="C6" s="8" t="inlineStr">
         <is>
@@ -804,7 +804,7 @@
         </is>
       </c>
       <c r="D6" s="7" t="n">
-        <v>5850</v>
+        <v>4500</v>
       </c>
       <c r="E6" s="9" t="inlineStr">
         <is>
@@ -815,11 +815,11 @@
     <row r="7" ht="16" customHeight="1">
       <c r="A7" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">  LVP installation — 2,340 SF @ $4.00/SF client price</t>
+          <t xml:space="preserve">  LVP installation — 1800 SF @ $4.00/SF client price</t>
         </is>
       </c>
       <c r="B7" s="11" t="n">
-        <v>6686</v>
+        <v>5143</v>
       </c>
       <c r="C7" s="12" t="inlineStr">
         <is>
@@ -827,7 +827,7 @@
         </is>
       </c>
       <c r="D7" s="11" t="n">
-        <v>9360</v>
+        <v>7200</v>
       </c>
       <c r="E7" s="13" t="inlineStr">
         <is>
@@ -884,11 +884,11 @@
         </is>
       </c>
       <c r="B10" s="16" t="n">
-        <v>13936</v>
+        <v>11043</v>
       </c>
       <c r="C10" s="15" t="n"/>
       <c r="D10" s="16" t="n">
-        <v>17170</v>
+        <v>13660</v>
       </c>
       <c r="E10" s="15" t="n"/>
     </row>
@@ -2110,6 +2110,17 @@
           <t xml:space="preserve">  Custom iron railing — upstairs back patio</t>
         </is>
       </c>
+      <c r="B86" t="n">
+        <v>2143</v>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>40%</t>
+        </is>
+      </c>
+      <c r="D86" t="n">
+        <v>3000</v>
+      </c>
     </row>
     <row r="87" ht="16" customHeight="1">
       <c r="A87" s="10" t="inlineStr">
@@ -2144,11 +2155,11 @@
         </is>
       </c>
       <c r="B89" s="16" t="n">
-        <v>857</v>
+        <v>3000</v>
       </c>
       <c r="C89" s="15" t="n"/>
       <c r="D89" s="16" t="n">
-        <v>1200</v>
+        <v>4200</v>
       </c>
       <c r="E89" s="15" t="n"/>
     </row>
@@ -2641,11 +2652,11 @@
         </is>
       </c>
       <c r="B128" s="40" t="n">
-        <v>114386</v>
+        <v>113636</v>
       </c>
       <c r="C128" s="40" t="n"/>
       <c r="D128" s="40" t="n">
-        <v>155481</v>
+        <v>154971</v>
       </c>
       <c r="E128" s="41" t="n"/>
     </row>
@@ -2659,7 +2670,7 @@
       <c r="B130" s="25" t="n"/>
       <c r="C130" s="25" t="n"/>
       <c r="D130" s="26" t="n">
-        <v>155481</v>
+        <v>154971</v>
       </c>
       <c r="E130" s="25" t="n"/>
     </row>
@@ -2670,7 +2681,7 @@
         </is>
       </c>
       <c r="D131" t="n">
-        <v>14383</v>
+        <v>14467</v>
       </c>
     </row>
     <row r="132" ht="16" customHeight="1">
@@ -2682,7 +2693,7 @@
       <c r="B132" s="29" t="n"/>
       <c r="C132" s="29" t="n"/>
       <c r="D132" s="30" t="n">
-        <v>41095</v>
+        <v>41335</v>
       </c>
       <c r="E132" s="29" t="n"/>
     </row>
@@ -2695,7 +2706,7 @@
       <c r="B133" s="25" t="n"/>
       <c r="C133" s="25" t="n"/>
       <c r="D133" s="26" t="n">
-        <v>26712</v>
+        <v>26868</v>
       </c>
       <c r="E133" s="25" t="n"/>
     </row>
@@ -2902,11 +2913,11 @@
         </is>
       </c>
       <c r="B146" s="36" t="n">
-        <v>138014</v>
+        <v>137264</v>
       </c>
       <c r="C146" s="35" t="n"/>
       <c r="D146" s="36" t="n">
-        <v>181441</v>
+        <v>180931</v>
       </c>
       <c r="E146" s="35" t="n"/>
     </row>

</xml_diff>

<commit_message>
Remove plumbing permit; new totals $154,371 / $180,331
</commit_message>
<xml_diff>
--- a/docs/san-palo-circle-robert-bird/San-Palo-Circle-Budget.xlsx
+++ b/docs/san-palo-circle-robert-bird/San-Palo-Circle-Budget.xlsx
@@ -2525,11 +2525,11 @@
         </is>
       </c>
       <c r="B119" s="40" t="n">
-        <v>6071</v>
+        <v>5643</v>
       </c>
       <c r="C119" s="40" t="n"/>
       <c r="D119" s="40" t="n">
-        <v>8500</v>
+        <v>7900</v>
       </c>
       <c r="E119" s="41" t="n"/>
     </row>
@@ -2652,11 +2652,11 @@
         </is>
       </c>
       <c r="B128" s="40" t="n">
-        <v>113636</v>
+        <v>113208</v>
       </c>
       <c r="C128" s="40" t="n"/>
       <c r="D128" s="40" t="n">
-        <v>154971</v>
+        <v>154371</v>
       </c>
       <c r="E128" s="41" t="n"/>
     </row>
@@ -2670,7 +2670,7 @@
       <c r="B130" s="25" t="n"/>
       <c r="C130" s="25" t="n"/>
       <c r="D130" s="26" t="n">
-        <v>154971</v>
+        <v>154371</v>
       </c>
       <c r="E130" s="25" t="n"/>
     </row>
@@ -2681,7 +2681,7 @@
         </is>
       </c>
       <c r="D131" t="n">
-        <v>14467</v>
+        <v>14407</v>
       </c>
     </row>
     <row r="132" ht="16" customHeight="1">
@@ -2693,7 +2693,7 @@
       <c r="B132" s="29" t="n"/>
       <c r="C132" s="29" t="n"/>
       <c r="D132" s="30" t="n">
-        <v>41335</v>
+        <v>41163</v>
       </c>
       <c r="E132" s="29" t="n"/>
     </row>
@@ -2706,7 +2706,7 @@
       <c r="B133" s="25" t="n"/>
       <c r="C133" s="25" t="n"/>
       <c r="D133" s="26" t="n">
-        <v>26868</v>
+        <v>26756</v>
       </c>
       <c r="E133" s="25" t="n"/>
     </row>
@@ -2917,7 +2917,7 @@
       </c>
       <c r="C146" s="35" t="n"/>
       <c r="D146" s="36" t="n">
-        <v>180931</v>
+        <v>180331</v>
       </c>
       <c r="E146" s="35" t="n"/>
     </row>

</xml_diff>

<commit_message>
Plumbing: excavation/relocation estimated at $3,500; new subtotal $5,600, project $152,071
</commit_message>
<xml_diff>
--- a/docs/san-palo-circle-robert-bird/San-Palo-Circle-Budget.xlsx
+++ b/docs/san-palo-circle-robert-bird/San-Palo-Circle-Budget.xlsx
@@ -2525,11 +2525,11 @@
         </is>
       </c>
       <c r="B119" s="40" t="n">
-        <v>5643</v>
+        <v>4000</v>
       </c>
       <c r="C119" s="40" t="n"/>
       <c r="D119" s="40" t="n">
-        <v>7900</v>
+        <v>5600</v>
       </c>
       <c r="E119" s="41" t="n"/>
     </row>
@@ -2652,11 +2652,11 @@
         </is>
       </c>
       <c r="B128" s="40" t="n">
-        <v>113208</v>
+        <v>111565</v>
       </c>
       <c r="C128" s="40" t="n"/>
       <c r="D128" s="40" t="n">
-        <v>154371</v>
+        <v>152071</v>
       </c>
       <c r="E128" s="41" t="n"/>
     </row>
@@ -2670,7 +2670,7 @@
       <c r="B130" s="25" t="n"/>
       <c r="C130" s="25" t="n"/>
       <c r="D130" s="26" t="n">
-        <v>154371</v>
+        <v>152071</v>
       </c>
       <c r="E130" s="25" t="n"/>
     </row>
@@ -2681,7 +2681,7 @@
         </is>
       </c>
       <c r="D131" t="n">
-        <v>14407</v>
+        <v>14177</v>
       </c>
     </row>
     <row r="132" ht="16" customHeight="1">
@@ -2693,7 +2693,7 @@
       <c r="B132" s="29" t="n"/>
       <c r="C132" s="29" t="n"/>
       <c r="D132" s="30" t="n">
-        <v>41163</v>
+        <v>40506</v>
       </c>
       <c r="E132" s="29" t="n"/>
     </row>
@@ -2706,7 +2706,7 @@
       <c r="B133" s="25" t="n"/>
       <c r="C133" s="25" t="n"/>
       <c r="D133" s="26" t="n">
-        <v>26756</v>
+        <v>26329</v>
       </c>
       <c r="E133" s="25" t="n"/>
     </row>
@@ -2917,7 +2917,7 @@
       </c>
       <c r="C146" s="35" t="n"/>
       <c r="D146" s="36" t="n">
-        <v>180331</v>
+        <v>178031</v>
       </c>
       <c r="E146" s="35" t="n"/>
     </row>

</xml_diff>

<commit_message>
Plumbing total $3,500 flat; project $149,971
</commit_message>
<xml_diff>
--- a/docs/san-palo-circle-robert-bird/San-Palo-Circle-Budget.xlsx
+++ b/docs/san-palo-circle-robert-bird/San-Palo-Circle-Budget.xlsx
@@ -2525,11 +2525,11 @@
         </is>
       </c>
       <c r="B119" s="40" t="n">
-        <v>4000</v>
+        <v>2500</v>
       </c>
       <c r="C119" s="40" t="n"/>
       <c r="D119" s="40" t="n">
-        <v>5600</v>
+        <v>3500</v>
       </c>
       <c r="E119" s="41" t="n"/>
     </row>
@@ -2652,11 +2652,11 @@
         </is>
       </c>
       <c r="B128" s="40" t="n">
-        <v>111565</v>
+        <v>110065</v>
       </c>
       <c r="C128" s="40" t="n"/>
       <c r="D128" s="40" t="n">
-        <v>152071</v>
+        <v>149971</v>
       </c>
       <c r="E128" s="41" t="n"/>
     </row>
@@ -2670,7 +2670,7 @@
       <c r="B130" s="25" t="n"/>
       <c r="C130" s="25" t="n"/>
       <c r="D130" s="26" t="n">
-        <v>152071</v>
+        <v>149971</v>
       </c>
       <c r="E130" s="25" t="n"/>
     </row>
@@ -2681,7 +2681,7 @@
         </is>
       </c>
       <c r="D131" t="n">
-        <v>14177</v>
+        <v>13967</v>
       </c>
     </row>
     <row r="132" ht="16" customHeight="1">
@@ -2693,7 +2693,7 @@
       <c r="B132" s="29" t="n"/>
       <c r="C132" s="29" t="n"/>
       <c r="D132" s="30" t="n">
-        <v>40506</v>
+        <v>39906</v>
       </c>
       <c r="E132" s="29" t="n"/>
     </row>
@@ -2706,7 +2706,7 @@
       <c r="B133" s="25" t="n"/>
       <c r="C133" s="25" t="n"/>
       <c r="D133" s="26" t="n">
-        <v>26329</v>
+        <v>25939</v>
       </c>
       <c r="E133" s="25" t="n"/>
     </row>
@@ -2917,7 +2917,7 @@
       </c>
       <c r="C146" s="35" t="n"/>
       <c r="D146" s="36" t="n">
-        <v>178031</v>
+        <v>175931</v>
       </c>
       <c r="E146" s="35" t="n"/>
     </row>

</xml_diff>

<commit_message>
Bathrooms: hot mop B1 walk-in, set new tub B2/B3, remove glass from tub baths; project $145,771
</commit_message>
<xml_diff>
--- a/docs/san-palo-circle-robert-bird/San-Palo-Circle-Budget.xlsx
+++ b/docs/san-palo-circle-robert-bird/San-Palo-Circle-Budget.xlsx
@@ -1452,11 +1452,11 @@
         </is>
       </c>
       <c r="B42" s="40" t="n">
-        <v>10150</v>
+        <v>9150</v>
       </c>
       <c r="C42" s="40" t="n"/>
       <c r="D42" s="40" t="n">
-        <v>13490</v>
+        <v>11390</v>
       </c>
       <c r="E42" s="41" t="n"/>
     </row>
@@ -1751,11 +1751,11 @@
         </is>
       </c>
       <c r="B58" s="16" t="n">
-        <v>9875</v>
+        <v>8875</v>
       </c>
       <c r="C58" s="15" t="n"/>
       <c r="D58" s="16" t="n">
-        <v>13105</v>
+        <v>11005</v>
       </c>
       <c r="E58" s="15" t="n"/>
     </row>
@@ -2652,11 +2652,11 @@
         </is>
       </c>
       <c r="B128" s="40" t="n">
-        <v>110065</v>
+        <v>108065</v>
       </c>
       <c r="C128" s="40" t="n"/>
       <c r="D128" s="40" t="n">
-        <v>149971</v>
+        <v>145771</v>
       </c>
       <c r="E128" s="41" t="n"/>
     </row>
@@ -2670,7 +2670,7 @@
       <c r="B130" s="25" t="n"/>
       <c r="C130" s="25" t="n"/>
       <c r="D130" s="26" t="n">
-        <v>149971</v>
+        <v>145771</v>
       </c>
       <c r="E130" s="25" t="n"/>
     </row>
@@ -2681,7 +2681,7 @@
         </is>
       </c>
       <c r="D131" t="n">
-        <v>13967</v>
+        <v>13547</v>
       </c>
     </row>
     <row r="132" ht="16" customHeight="1">
@@ -2693,7 +2693,7 @@
       <c r="B132" s="29" t="n"/>
       <c r="C132" s="29" t="n"/>
       <c r="D132" s="30" t="n">
-        <v>39906</v>
+        <v>37706</v>
       </c>
       <c r="E132" s="29" t="n"/>
     </row>
@@ -2706,7 +2706,7 @@
       <c r="B133" s="25" t="n"/>
       <c r="C133" s="25" t="n"/>
       <c r="D133" s="26" t="n">
-        <v>25939</v>
+        <v>24159</v>
       </c>
       <c r="E133" s="25" t="n"/>
     </row>
@@ -2917,7 +2917,7 @@
       </c>
       <c r="C146" s="35" t="n"/>
       <c r="D146" s="36" t="n">
-        <v>175931</v>
+        <v>171731</v>
       </c>
       <c r="E146" s="35" t="n"/>
     </row>

</xml_diff>